<commit_message>
impute works with vector of variables; method selected from dt_meta if NULL; tidying
</commit_message>
<xml_diff>
--- a/tests/testthat/data-raw/dt_meta.xlsx
+++ b/tests/testthat/data-raw/dt_meta.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\plevy\Documents\metamet\tests\testthat\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\plevy\Documents\metamet\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708A3F8C-FC06-459C-884D-3F89252C3824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EFF005F-4CCA-4AE3-8886-42E2399916F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
   </bookViews>
   <sheets>
     <sheet name="dt_meta" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1329" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="235">
   <si>
     <t>name_dt</t>
   </si>
@@ -794,12 +794,24 @@
   <si>
     <t>mm</t>
   </si>
+  <si>
+    <t>imputation_method</t>
+  </si>
+  <si>
+    <t>era5</t>
+  </si>
+  <si>
+    <t>zero</t>
+  </si>
+  <si>
+    <t>nightzero</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -930,6 +942,12 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1663,7 +1681,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B621CE1-A4D4-4502-917D-92507EE2F7EE}">
-  <dimension ref="A1:V104"/>
+  <dimension ref="A1:W104"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -1673,7 +1691,7 @@
     <col min="8" max="9" width="15.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>117</v>
       </c>
@@ -1740,8 +1758,11 @@
       <c r="V1" s="2" t="s">
         <v>226</v>
       </c>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W1" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>118</v>
       </c>
@@ -1807,8 +1828,11 @@
         <f>VLOOKUP($C2,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>NA</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W2" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>118</v>
       </c>
@@ -1876,8 +1900,11 @@
         <f>VLOOKUP($C3,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>cm</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W3" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>118</v>
       </c>
@@ -1945,8 +1972,11 @@
         <f>VLOOKUP($C4,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>cm</v>
       </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W4" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>118</v>
       </c>
@@ -2014,8 +2044,11 @@
         <f>VLOOKUP($C5,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>NA</v>
       </c>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W5" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>118</v>
       </c>
@@ -2083,8 +2116,11 @@
         <f>VLOOKUP($C6,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W6" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>118</v>
       </c>
@@ -2152,8 +2188,11 @@
         <f>VLOOKUP($C7,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W7" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>118</v>
       </c>
@@ -2221,8 +2260,11 @@
         <f>VLOOKUP($C8,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W8" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>118</v>
       </c>
@@ -2290,8 +2332,11 @@
         <f>VLOOKUP($C9,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W9" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>118</v>
       </c>
@@ -2359,8 +2404,11 @@
         <f>VLOOKUP($C10,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W10" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>118</v>
       </c>
@@ -2428,8 +2476,11 @@
         <f>VLOOKUP($C11,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W11" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>118</v>
       </c>
@@ -2497,8 +2548,11 @@
         <f>VLOOKUP($C12,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W12" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>118</v>
       </c>
@@ -2566,8 +2620,11 @@
         <f>VLOOKUP($C13,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W13" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>118</v>
       </c>
@@ -2635,8 +2692,11 @@
         <f>VLOOKUP($C14,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>1</v>
       </c>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W14" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>118</v>
       </c>
@@ -2704,8 +2764,11 @@
         <f>VLOOKUP($C15,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W15" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>118</v>
       </c>
@@ -2773,8 +2836,11 @@
         <f>VLOOKUP($C16,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W16" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>118</v>
       </c>
@@ -2842,8 +2908,11 @@
         <f>VLOOKUP($C17,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W17" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>118</v>
       </c>
@@ -2911,8 +2980,11 @@
         <f>VLOOKUP($C18,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W18" s="2" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>118</v>
       </c>
@@ -2980,8 +3052,11 @@
         <f>VLOOKUP($C19,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>mm</v>
       </c>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W19" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>118</v>
       </c>
@@ -3049,8 +3124,11 @@
         <f>VLOOKUP($C20,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>mm</v>
       </c>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W20" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>118</v>
       </c>
@@ -3118,8 +3196,11 @@
         <f>VLOOKUP($C21,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>kPa</v>
       </c>
-    </row>
-    <row r="22" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W21" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>118</v>
       </c>
@@ -3187,8 +3268,11 @@
         <f>VLOOKUP($C22,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="23" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W22" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>118</v>
       </c>
@@ -3256,8 +3340,11 @@
         <f>VLOOKUP($C23,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="24" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W23" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>118</v>
       </c>
@@ -3325,8 +3412,11 @@
         <f>VLOOKUP($C24,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="25" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W24" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>118</v>
       </c>
@@ -3394,8 +3484,11 @@
         <f>VLOOKUP($C25,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="26" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W25" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>118</v>
       </c>
@@ -3463,8 +3556,11 @@
         <f>VLOOKUP($C26,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="27" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W26" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>118</v>
       </c>
@@ -3532,8 +3628,11 @@
         <f>VLOOKUP($C27,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="28" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W27" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>118</v>
       </c>
@@ -3601,8 +3700,11 @@
         <f>VLOOKUP($C28,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>micromol / m^2 / s</v>
       </c>
-    </row>
-    <row r="29" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W28" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>118</v>
       </c>
@@ -3670,8 +3772,11 @@
         <f>VLOOKUP($C29,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="30" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W29" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>118</v>
       </c>
@@ -3740,8 +3845,11 @@
         <f>VLOOKUP($C30,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="31" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W30" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>118</v>
       </c>
@@ -3810,8 +3918,11 @@
         <f>VLOOKUP($C31,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="32" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W31" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>118</v>
       </c>
@@ -3880,8 +3991,11 @@
         <f>VLOOKUP($C32,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="33" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W32" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>118</v>
       </c>
@@ -3950,8 +4064,11 @@
         <f>VLOOKUP($C33,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="34" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W33" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>118</v>
       </c>
@@ -4019,8 +4136,11 @@
         <f>VLOOKUP($C34,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="35" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W34" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>118</v>
       </c>
@@ -4089,8 +4209,11 @@
         <f>VLOOKUP($C35,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="36" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W35" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>118</v>
       </c>
@@ -4159,8 +4282,11 @@
         <f>VLOOKUP($C36,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="37" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W36" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>118</v>
       </c>
@@ -4228,8 +4354,11 @@
         <f>VLOOKUP($C37,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="38" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W37" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>118</v>
       </c>
@@ -4297,8 +4426,11 @@
         <f>VLOOKUP($C38,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="39" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W38" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>118</v>
       </c>
@@ -4366,8 +4498,11 @@
         <f>VLOOKUP($C39,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="40" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W39" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>118</v>
       </c>
@@ -4436,8 +4571,11 @@
         <f>VLOOKUP($C40,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="41" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W40" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>118</v>
       </c>
@@ -4506,8 +4644,11 @@
         <f>VLOOKUP($C41,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="42" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W41" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>118</v>
       </c>
@@ -4576,8 +4717,11 @@
         <f>VLOOKUP($C42,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="43" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W42" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>118</v>
       </c>
@@ -4646,8 +4790,11 @@
         <f>VLOOKUP($C43,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="44" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W43" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>118</v>
       </c>
@@ -4716,8 +4863,11 @@
         <f>VLOOKUP($C44,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="45" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W44" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>118</v>
       </c>
@@ -4786,8 +4936,11 @@
         <f>VLOOKUP($C45,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="46" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W45" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>118</v>
       </c>
@@ -4856,8 +5009,11 @@
         <f>VLOOKUP($C46,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="47" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W46" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>118</v>
       </c>
@@ -4925,8 +5081,11 @@
         <f>VLOOKUP($C47,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>NA</v>
       </c>
-    </row>
-    <row r="48" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W47" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>118</v>
       </c>
@@ -4995,8 +5154,11 @@
         <f>VLOOKUP($C48,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree</v>
       </c>
-    </row>
-    <row r="49" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W48" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>118</v>
       </c>
@@ -5065,8 +5227,11 @@
         <f>VLOOKUP($C49,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>m / s</v>
       </c>
-    </row>
-    <row r="50" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W49" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>118</v>
       </c>
@@ -5135,8 +5300,11 @@
         <f>VLOOKUP($C50,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree</v>
       </c>
-    </row>
-    <row r="51" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W50" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>118</v>
       </c>
@@ -5205,8 +5373,11 @@
         <f>VLOOKUP($C51,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>m / s</v>
       </c>
-    </row>
-    <row r="52" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W51" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>118</v>
       </c>
@@ -5274,8 +5445,11 @@
         <f>VLOOKUP($C52,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>m</v>
       </c>
-    </row>
-    <row r="53" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W52" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>118</v>
       </c>
@@ -5343,8 +5517,11 @@
         <f>VLOOKUP($C53,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>m</v>
       </c>
-    </row>
-    <row r="54" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W53" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>118</v>
       </c>
@@ -5412,8 +5589,11 @@
         <f>VLOOKUP($C54,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="55" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W54" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>118</v>
       </c>
@@ -5481,8 +5661,11 @@
         <f>VLOOKUP($C55,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="56" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W55" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>118</v>
       </c>
@@ -5550,8 +5733,11 @@
         <f>VLOOKUP($C56,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="57" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W56" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>118</v>
       </c>
@@ -5619,8 +5805,11 @@
         <f>VLOOKUP($C57,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="58" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W57" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>118</v>
       </c>
@@ -5688,8 +5877,11 @@
         <f>VLOOKUP($C58,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="59" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W58" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>118</v>
       </c>
@@ -5758,8 +5950,11 @@
         <f>VLOOKUP($C59,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="60" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W59" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>118</v>
       </c>
@@ -5828,8 +6023,11 @@
         <f>VLOOKUP($C60,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="61" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W60" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>118</v>
       </c>
@@ -5898,8 +6096,11 @@
         <f>VLOOKUP($C61,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="62" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W61" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>118</v>
       </c>
@@ -5968,8 +6169,11 @@
         <f>VLOOKUP($C62,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="63" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W62" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>118</v>
       </c>
@@ -6038,8 +6242,11 @@
         <f>VLOOKUP($C63,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="64" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W63" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="64" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>118</v>
       </c>
@@ -6108,8 +6315,11 @@
         <f>VLOOKUP($C64,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="65" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W64" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="65" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>118</v>
       </c>
@@ -6178,8 +6388,11 @@
         <f>VLOOKUP($C65,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="66" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W65" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="66" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>118</v>
       </c>
@@ -6248,8 +6461,11 @@
         <f>VLOOKUP($C66,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="67" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W66" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="67" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>118</v>
       </c>
@@ -6318,8 +6534,11 @@
         <f>VLOOKUP($C67,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="68" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W67" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="68" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>118</v>
       </c>
@@ -6388,8 +6607,11 @@
         <f>VLOOKUP($C68,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="69" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W68" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="69" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>118</v>
       </c>
@@ -6458,8 +6680,11 @@
         <f>VLOOKUP($C69,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="70" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W69" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="70" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>118</v>
       </c>
@@ -6528,8 +6753,11 @@
         <f>VLOOKUP($C70,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="71" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W70" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="71" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>118</v>
       </c>
@@ -6598,8 +6826,11 @@
         <f>VLOOKUP($C71,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="72" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W71" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="72" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>118</v>
       </c>
@@ -6668,8 +6899,11 @@
         <f>VLOOKUP($C72,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>W / m^2</v>
       </c>
-    </row>
-    <row r="73" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W72" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="73" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>118</v>
       </c>
@@ -6738,8 +6972,11 @@
         <f>VLOOKUP($C73,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>m</v>
       </c>
-    </row>
-    <row r="74" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W73" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="74" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>118</v>
       </c>
@@ -6808,8 +7045,11 @@
         <f>VLOOKUP($C74,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>m</v>
       </c>
-    </row>
-    <row r="75" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W74" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="75" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>118</v>
       </c>
@@ -6878,8 +7118,11 @@
         <f>VLOOKUP($C75,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>m</v>
       </c>
-    </row>
-    <row r="76" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W75" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="76" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>118</v>
       </c>
@@ -6948,8 +7191,11 @@
         <f>VLOOKUP($C76,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>m</v>
       </c>
-    </row>
-    <row r="77" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W76" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="77" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>118</v>
       </c>
@@ -7018,8 +7264,11 @@
         <f>VLOOKUP($C77,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="78" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W77" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="78" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>118</v>
       </c>
@@ -7088,8 +7337,11 @@
         <f>VLOOKUP($C78,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="79" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W78" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="79" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>118</v>
       </c>
@@ -7158,8 +7410,11 @@
         <f>VLOOKUP($C79,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="80" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W79" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="80" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>118</v>
       </c>
@@ -7228,8 +7483,11 @@
         <f>VLOOKUP($C80,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="81" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W80" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="81" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>118</v>
       </c>
@@ -7298,8 +7556,11 @@
         <f>VLOOKUP($C81,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="82" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W81" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="82" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>118</v>
       </c>
@@ -7368,8 +7629,11 @@
         <f>VLOOKUP($C82,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="83" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W82" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="83" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>118</v>
       </c>
@@ -7438,8 +7702,11 @@
         <f>VLOOKUP($C83,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="84" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W83" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="84" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>118</v>
       </c>
@@ -7508,8 +7775,11 @@
         <f>VLOOKUP($C84,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="85" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W84" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="85" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>118</v>
       </c>
@@ -7578,8 +7848,11 @@
         <f>VLOOKUP($C85,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="86" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W85" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="86" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>118</v>
       </c>
@@ -7648,8 +7921,11 @@
         <f>VLOOKUP($C86,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="87" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W86" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="87" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>118</v>
       </c>
@@ -7718,8 +7994,11 @@
         <f>VLOOKUP($C87,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="88" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W87" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="88" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>118</v>
       </c>
@@ -7788,8 +8067,11 @@
         <f>VLOOKUP($C88,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="89" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W88" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="89" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>118</v>
       </c>
@@ -7858,8 +8140,11 @@
         <f>VLOOKUP($C89,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="90" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W89" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="90" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>118</v>
       </c>
@@ -7928,8 +8213,11 @@
         <f>VLOOKUP($C90,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="91" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W90" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="91" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>118</v>
       </c>
@@ -7998,8 +8286,11 @@
         <f>VLOOKUP($C91,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="92" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W91" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="92" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>118</v>
       </c>
@@ -8068,8 +8359,11 @@
         <f>VLOOKUP($C92,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="93" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W92" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="93" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>118</v>
       </c>
@@ -8138,8 +8432,11 @@
         <f>VLOOKUP($C93,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="94" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W93" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="94" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>118</v>
       </c>
@@ -8208,8 +8505,11 @@
         <f>VLOOKUP($C94,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="95" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W94" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="95" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>118</v>
       </c>
@@ -8278,8 +8578,11 @@
         <f>VLOOKUP($C95,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="96" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W95" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="96" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>118</v>
       </c>
@@ -8348,8 +8651,11 @@
         <f>VLOOKUP($C96,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="97" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W96" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="97" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>118</v>
       </c>
@@ -8418,8 +8724,11 @@
         <f>VLOOKUP($C97,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="98" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W97" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="98" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>118</v>
       </c>
@@ -8488,8 +8797,11 @@
         <f>VLOOKUP($C98,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="99" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W98" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="99" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>118</v>
       </c>
@@ -8558,8 +8870,11 @@
         <f>VLOOKUP($C99,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="100" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W99" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="100" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>118</v>
       </c>
@@ -8628,8 +8943,11 @@
         <f>VLOOKUP($C100,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="101" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W100" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="101" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>118</v>
       </c>
@@ -8698,8 +9016,11 @@
         <f>VLOOKUP($C101,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="102" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W101" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="102" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>118</v>
       </c>
@@ -8768,8 +9089,11 @@
         <f>VLOOKUP($C102,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>percent</v>
       </c>
-    </row>
-    <row r="103" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W102" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="103" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>119</v>
       </c>
@@ -8838,8 +9162,11 @@
         <f>VLOOKUP($C103,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-    </row>
-    <row r="104" spans="1:22" x14ac:dyDescent="0.3">
+      <c r="W103" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="104" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>120</v>
       </c>
@@ -8907,12 +9234,16 @@
       <c r="V104" t="str">
         <f>VLOOKUP($C104,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
+      </c>
+      <c r="W104" s="2" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B3:R53">
     <sortCondition ref="B3:B53"/>
   </sortState>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="120" verticalDpi="72" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
added Whim test; fixed arising bugs
</commit_message>
<xml_diff>
--- a/tests/testthat/data-raw/dt_meta.xlsx
+++ b/tests/testthat/data-raw/dt_meta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\plevy\Documents\metamet\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EFF005F-4CCA-4AE3-8886-42E2399916F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD8B3D4E-CA64-4C16-8CA6-056653E8E9C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
   </bookViews>
   <sheets>
     <sheet name="dt_meta" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1606" uniqueCount="247">
   <si>
     <t>name_dt</t>
   </si>
@@ -805,6 +805,42 @@
   </si>
   <si>
     <t>nightzero</t>
+  </si>
+  <si>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>Rain</t>
+  </si>
+  <si>
+    <t>AirT</t>
+  </si>
+  <si>
+    <t>PAR</t>
+  </si>
+  <si>
+    <t>Total_solar</t>
+  </si>
+  <si>
+    <t>Net_rad</t>
+  </si>
+  <si>
+    <t>Soil_VWC</t>
+  </si>
+  <si>
+    <t>Soil_T1</t>
+  </si>
+  <si>
+    <t>Soil_T2</t>
+  </si>
+  <si>
+    <t>Shortwave incoming radiation</t>
+  </si>
+  <si>
+    <t>Shortwave outgoing radiation</t>
+  </si>
+  <si>
+    <t>%d/%m/%Y %H:%M</t>
   </si>
 </sst>
 </file>
@@ -1681,7 +1717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B621CE1-A4D4-4502-917D-92507EE2F7EE}">
-  <dimension ref="A1:W104"/>
+  <dimension ref="A1:W118"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
@@ -4078,8 +4114,8 @@
       <c r="C34" t="s">
         <v>36</v>
       </c>
-      <c r="D34" t="s">
-        <v>37</v>
+      <c r="D34" s="2" t="s">
+        <v>244</v>
       </c>
       <c r="E34" t="s">
         <v>27</v>
@@ -4152,7 +4188,7 @@
         <v>36</v>
       </c>
       <c r="D35" t="s">
-        <v>37</v>
+        <v>244</v>
       </c>
       <c r="E35" t="s">
         <v>27</v>
@@ -4225,7 +4261,7 @@
         <v>36</v>
       </c>
       <c r="D36" t="s">
-        <v>37</v>
+        <v>244</v>
       </c>
       <c r="E36" t="s">
         <v>27</v>
@@ -4297,7 +4333,7 @@
         <v>38</v>
       </c>
       <c r="D37" t="s">
-        <v>39</v>
+        <v>245</v>
       </c>
       <c r="E37" t="s">
         <v>27</v>
@@ -4369,7 +4405,7 @@
         <v>38</v>
       </c>
       <c r="D38" t="s">
-        <v>39</v>
+        <v>245</v>
       </c>
       <c r="E38" t="s">
         <v>27</v>
@@ -9170,36 +9206,35 @@
       <c r="A104" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B104" s="2" t="str">
-        <f t="shared" ref="B104" si="13">C104&amp;"_"&amp;J104&amp;"_"&amp;K104&amp;"_"&amp;L104</f>
-        <v>TA_2_1_1</v>
+      <c r="B104" t="s">
+        <v>117</v>
       </c>
       <c r="C104" t="s">
-        <v>72</v>
+        <v>117</v>
       </c>
       <c r="D104" t="s">
-        <v>73</v>
+        <v>117</v>
       </c>
       <c r="E104" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F104" t="s">
-        <v>103</v>
+        <v>117</v>
       </c>
       <c r="H104" s="1">
-        <v>46023</v>
+        <v>37257</v>
       </c>
       <c r="I104" s="1">
-        <v>46388</v>
-      </c>
-      <c r="J104">
-        <v>2</v>
-      </c>
-      <c r="K104">
-        <v>1</v>
-      </c>
-      <c r="L104">
-        <v>1</v>
+        <v>47484</v>
+      </c>
+      <c r="J104" t="s">
+        <v>16</v>
+      </c>
+      <c r="K104" t="s">
+        <v>16</v>
+      </c>
+      <c r="L104" t="s">
+        <v>16</v>
       </c>
       <c r="M104" t="b">
         <v>0</v>
@@ -9219,23 +9254,1034 @@
       <c r="R104" t="s">
         <v>21</v>
       </c>
-      <c r="S104">
+      <c r="S104" t="e">
         <f>VLOOKUP($C104,naming_lookup!$C$1:$H$40,3,FALSE)</f>
-        <v>-40</v>
-      </c>
-      <c r="T104">
+        <v>#N/A</v>
+      </c>
+      <c r="T104" t="e">
         <f>VLOOKUP($C104,naming_lookup!$C$1:$H$40,4,FALSE)</f>
-        <v>50</v>
+        <v>#N/A</v>
       </c>
       <c r="U104" t="str">
         <f>VLOOKUP($C104,naming_lookup!$C$1:$H$40,5,FALSE)</f>
-        <v>t2m</v>
+        <v>site</v>
       </c>
       <c r="V104" t="str">
         <f>VLOOKUP($C104,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>NA</v>
+      </c>
+      <c r="W104" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="105" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A105" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B105" t="s">
+        <v>235</v>
+      </c>
+      <c r="C105" t="s">
+        <v>15</v>
+      </c>
+      <c r="D105" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="E105" t="s">
+        <v>16</v>
+      </c>
+      <c r="F105" t="s">
+        <v>97</v>
+      </c>
+      <c r="G105" s="2" t="s">
+        <v>246</v>
+      </c>
+      <c r="H105" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I105" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J105" t="s">
+        <v>16</v>
+      </c>
+      <c r="K105" t="s">
+        <v>16</v>
+      </c>
+      <c r="L105" t="s">
+        <v>16</v>
+      </c>
+      <c r="M105" t="b">
+        <v>0</v>
+      </c>
+      <c r="N105" t="b">
+        <v>1</v>
+      </c>
+      <c r="O105" t="b">
+        <v>0</v>
+      </c>
+      <c r="P105">
+        <v>100</v>
+      </c>
+      <c r="Q105" t="s">
+        <v>20</v>
+      </c>
+      <c r="R105" t="s">
+        <v>21</v>
+      </c>
+      <c r="S105">
+        <f>VLOOKUP($C105,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="T105">
+        <f>VLOOKUP($C105,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="U105" t="str">
+        <f>VLOOKUP($C105,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>time</v>
+      </c>
+      <c r="V105" t="str">
+        <f>VLOOKUP($C105,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>NA</v>
+      </c>
+      <c r="W105" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="106" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A106" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B106" t="s">
+        <v>236</v>
+      </c>
+      <c r="C106" t="s">
+        <v>53</v>
+      </c>
+      <c r="D106" t="s">
+        <v>54</v>
+      </c>
+      <c r="E106" t="s">
+        <v>230</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="H106" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I106" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J106" t="s">
+        <v>16</v>
+      </c>
+      <c r="K106" t="s">
+        <v>16</v>
+      </c>
+      <c r="L106" t="s">
+        <v>16</v>
+      </c>
+      <c r="M106" t="b">
+        <v>0</v>
+      </c>
+      <c r="N106" t="b">
+        <v>1</v>
+      </c>
+      <c r="O106" t="b">
+        <v>0</v>
+      </c>
+      <c r="P106">
+        <v>100</v>
+      </c>
+      <c r="Q106" t="s">
+        <v>20</v>
+      </c>
+      <c r="R106" t="s">
+        <v>21</v>
+      </c>
+      <c r="S106">
+        <f>VLOOKUP($C106,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="T106">
+        <f>VLOOKUP($C106,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="U106" t="str">
+        <f>VLOOKUP($C106,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>tp</v>
+      </c>
+      <c r="V106" t="str">
+        <f>VLOOKUP($C106,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>mm</v>
+      </c>
+      <c r="W106" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="107" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A107" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B107" t="s">
+        <v>152</v>
+      </c>
+      <c r="C107" t="s">
+        <v>152</v>
+      </c>
+      <c r="D107" t="s">
+        <v>87</v>
+      </c>
+      <c r="E107" t="s">
+        <v>88</v>
+      </c>
+      <c r="F107" t="s">
+        <v>99</v>
+      </c>
+      <c r="H107" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I107" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J107" t="s">
+        <v>16</v>
+      </c>
+      <c r="K107" t="s">
+        <v>16</v>
+      </c>
+      <c r="L107" t="s">
+        <v>16</v>
+      </c>
+      <c r="M107" t="b">
+        <v>0</v>
+      </c>
+      <c r="N107" t="b">
+        <v>1</v>
+      </c>
+      <c r="O107" t="b">
+        <v>0</v>
+      </c>
+      <c r="P107">
+        <v>100</v>
+      </c>
+      <c r="Q107" t="s">
+        <v>20</v>
+      </c>
+      <c r="R107" t="s">
+        <v>21</v>
+      </c>
+      <c r="S107">
+        <f>VLOOKUP($C107,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-99999</v>
+      </c>
+      <c r="T107">
+        <f>VLOOKUP($C107,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>99999</v>
+      </c>
+      <c r="U107" t="str">
+        <f>VLOOKUP($C107,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>rh</v>
+      </c>
+      <c r="V107">
+        <f>VLOOKUP($C107,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="W107" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="108" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A108" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B108" t="s">
+        <v>237</v>
+      </c>
+      <c r="C108" t="s">
+        <v>72</v>
+      </c>
+      <c r="D108" t="s">
+        <v>73</v>
+      </c>
+      <c r="E108" t="s">
+        <v>191</v>
+      </c>
+      <c r="F108" t="s">
+        <v>103</v>
+      </c>
+      <c r="H108" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I108" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J108" t="s">
+        <v>16</v>
+      </c>
+      <c r="K108" t="s">
+        <v>16</v>
+      </c>
+      <c r="L108" t="s">
+        <v>16</v>
+      </c>
+      <c r="M108" t="b">
+        <v>0</v>
+      </c>
+      <c r="N108" t="b">
+        <v>1</v>
+      </c>
+      <c r="O108" t="b">
+        <v>0</v>
+      </c>
+      <c r="P108">
+        <v>100</v>
+      </c>
+      <c r="Q108" t="s">
+        <v>20</v>
+      </c>
+      <c r="R108" t="s">
+        <v>21</v>
+      </c>
+      <c r="S108">
+        <f>VLOOKUP($C108,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-40</v>
+      </c>
+      <c r="T108">
+        <f>VLOOKUP($C108,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="U108" t="str">
+        <f>VLOOKUP($C108,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>t2m</v>
+      </c>
+      <c r="V108" t="str">
+        <f>VLOOKUP($C108,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-      <c r="W104" s="2" t="s">
+      <c r="W108" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="109" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A109" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B109" t="s">
+        <v>74</v>
+      </c>
+      <c r="C109" t="s">
+        <v>74</v>
+      </c>
+      <c r="D109" t="s">
+        <v>75</v>
+      </c>
+      <c r="E109" t="s">
+        <v>175</v>
+      </c>
+      <c r="F109" t="s">
+        <v>101</v>
+      </c>
+      <c r="H109" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I109" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J109" t="s">
+        <v>16</v>
+      </c>
+      <c r="K109" t="s">
+        <v>16</v>
+      </c>
+      <c r="L109" t="s">
+        <v>16</v>
+      </c>
+      <c r="M109" t="b">
+        <v>0</v>
+      </c>
+      <c r="N109" t="b">
+        <v>1</v>
+      </c>
+      <c r="O109" t="b">
+        <v>0</v>
+      </c>
+      <c r="P109">
+        <v>100</v>
+      </c>
+      <c r="Q109" t="s">
+        <v>20</v>
+      </c>
+      <c r="R109" t="s">
+        <v>21</v>
+      </c>
+      <c r="S109">
+        <f>VLOOKUP($C109,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>30</v>
+      </c>
+      <c r="T109">
+        <f>VLOOKUP($C109,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>120</v>
+      </c>
+      <c r="U109" t="str">
+        <f>VLOOKUP($C109,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>rh</v>
+      </c>
+      <c r="V109" t="str">
+        <f>VLOOKUP($C109,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>percent</v>
+      </c>
+      <c r="W109" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="110" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A110" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B110" t="s">
+        <v>238</v>
+      </c>
+      <c r="C110" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D110" t="s">
+        <v>46</v>
+      </c>
+      <c r="E110" t="s">
+        <v>155</v>
+      </c>
+      <c r="F110" t="s">
+        <v>98</v>
+      </c>
+      <c r="H110" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I110" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J110" t="s">
+        <v>16</v>
+      </c>
+      <c r="K110" t="s">
+        <v>16</v>
+      </c>
+      <c r="L110" t="s">
+        <v>16</v>
+      </c>
+      <c r="M110" t="b">
+        <v>0</v>
+      </c>
+      <c r="N110" t="b">
+        <v>1</v>
+      </c>
+      <c r="O110" t="b">
+        <v>0</v>
+      </c>
+      <c r="P110">
+        <v>100</v>
+      </c>
+      <c r="Q110" t="s">
+        <v>20</v>
+      </c>
+      <c r="R110" t="s">
+        <v>21</v>
+      </c>
+      <c r="S110">
+        <f>VLOOKUP($C110,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="T110">
+        <f>VLOOKUP($C110,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>2200</v>
+      </c>
+      <c r="U110" t="str">
+        <f>VLOOKUP($C110,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="V110" t="str">
+        <f>VLOOKUP($C110,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>micromol / m^2 / s</v>
+      </c>
+      <c r="W110" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="111" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A111" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B111" t="s">
+        <v>239</v>
+      </c>
+      <c r="C111" t="s">
+        <v>36</v>
+      </c>
+      <c r="D111" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E111" t="s">
+        <v>142</v>
+      </c>
+      <c r="F111" t="s">
+        <v>98</v>
+      </c>
+      <c r="H111" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I111" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J111" t="s">
+        <v>16</v>
+      </c>
+      <c r="K111" t="s">
+        <v>16</v>
+      </c>
+      <c r="L111" t="s">
+        <v>16</v>
+      </c>
+      <c r="M111" t="b">
+        <v>0</v>
+      </c>
+      <c r="N111" t="b">
+        <v>1</v>
+      </c>
+      <c r="O111" t="b">
+        <v>0</v>
+      </c>
+      <c r="P111">
+        <v>100</v>
+      </c>
+      <c r="Q111" t="s">
+        <v>20</v>
+      </c>
+      <c r="R111" t="s">
+        <v>21</v>
+      </c>
+      <c r="S111">
+        <f>VLOOKUP($C111,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="T111">
+        <f>VLOOKUP($C111,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>1200</v>
+      </c>
+      <c r="U111" t="str">
+        <f>VLOOKUP($C111,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="V111" t="str">
+        <f>VLOOKUP($C111,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>W / m^2</v>
+      </c>
+      <c r="W111" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="112" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A112" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B112" t="s">
+        <v>240</v>
+      </c>
+      <c r="C112" t="s">
+        <v>114</v>
+      </c>
+      <c r="D112" t="s">
+        <v>65</v>
+      </c>
+      <c r="E112" t="s">
+        <v>142</v>
+      </c>
+      <c r="F112" t="s">
+        <v>98</v>
+      </c>
+      <c r="H112" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I112" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J112" t="s">
+        <v>16</v>
+      </c>
+      <c r="K112" t="s">
+        <v>16</v>
+      </c>
+      <c r="L112" t="s">
+        <v>16</v>
+      </c>
+      <c r="M112" t="b">
+        <v>0</v>
+      </c>
+      <c r="N112" t="b">
+        <v>1</v>
+      </c>
+      <c r="O112" t="b">
+        <v>0</v>
+      </c>
+      <c r="P112">
+        <v>100</v>
+      </c>
+      <c r="Q112" t="s">
+        <v>20</v>
+      </c>
+      <c r="R112" t="s">
+        <v>21</v>
+      </c>
+      <c r="S112">
+        <f>VLOOKUP($C112,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-500</v>
+      </c>
+      <c r="T112">
+        <f>VLOOKUP($C112,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>1200</v>
+      </c>
+      <c r="U112" t="str">
+        <f>VLOOKUP($C112,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>rn</v>
+      </c>
+      <c r="V112" t="str">
+        <f>VLOOKUP($C112,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>W / m^2</v>
+      </c>
+      <c r="W112" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="113" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A113" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B113" t="s">
+        <v>56</v>
+      </c>
+      <c r="C113" t="s">
+        <v>56</v>
+      </c>
+      <c r="D113" t="s">
+        <v>57</v>
+      </c>
+      <c r="E113" t="s">
+        <v>229</v>
+      </c>
+      <c r="F113" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H113" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I113" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J113" t="s">
+        <v>16</v>
+      </c>
+      <c r="K113" t="s">
+        <v>16</v>
+      </c>
+      <c r="L113" t="s">
+        <v>16</v>
+      </c>
+      <c r="M113" t="b">
+        <v>0</v>
+      </c>
+      <c r="N113" t="b">
+        <v>1</v>
+      </c>
+      <c r="O113" t="b">
+        <v>0</v>
+      </c>
+      <c r="P113">
+        <v>100</v>
+      </c>
+      <c r="Q113" t="s">
+        <v>20</v>
+      </c>
+      <c r="R113" t="s">
+        <v>21</v>
+      </c>
+      <c r="S113">
+        <f>VLOOKUP($C113,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="T113">
+        <f>VLOOKUP($C113,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>30</v>
+      </c>
+      <c r="U113" t="str">
+        <f>VLOOKUP($C113,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ws</v>
+      </c>
+      <c r="V113" t="str">
+        <f>VLOOKUP($C113,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>m / s</v>
+      </c>
+      <c r="W113" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="114" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A114" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B114" t="s">
+        <v>59</v>
+      </c>
+      <c r="C114" t="s">
+        <v>59</v>
+      </c>
+      <c r="D114" t="s">
+        <v>60</v>
+      </c>
+      <c r="E114" t="s">
+        <v>198</v>
+      </c>
+      <c r="F114" t="s">
+        <v>105</v>
+      </c>
+      <c r="H114" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I114" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J114" t="s">
+        <v>16</v>
+      </c>
+      <c r="K114" t="s">
+        <v>16</v>
+      </c>
+      <c r="L114" t="s">
+        <v>16</v>
+      </c>
+      <c r="M114" t="b">
+        <v>0</v>
+      </c>
+      <c r="N114" t="b">
+        <v>1</v>
+      </c>
+      <c r="O114" t="b">
+        <v>0</v>
+      </c>
+      <c r="P114">
+        <v>100</v>
+      </c>
+      <c r="Q114" t="s">
+        <v>20</v>
+      </c>
+      <c r="R114" t="s">
+        <v>21</v>
+      </c>
+      <c r="S114">
+        <f>VLOOKUP($C114,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="T114">
+        <f>VLOOKUP($C114,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>360</v>
+      </c>
+      <c r="U114" t="str">
+        <f>VLOOKUP($C114,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>wd</v>
+      </c>
+      <c r="V114" t="str">
+        <f>VLOOKUP($C114,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>degree</v>
+      </c>
+      <c r="W114" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="115" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A115" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B115" t="s">
+        <v>241</v>
+      </c>
+      <c r="C115" t="s">
+        <v>22</v>
+      </c>
+      <c r="D115" t="s">
+        <v>23</v>
+      </c>
+      <c r="E115" t="s">
+        <v>175</v>
+      </c>
+      <c r="F115" t="s">
+        <v>102</v>
+      </c>
+      <c r="H115" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I115" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J115" t="s">
+        <v>16</v>
+      </c>
+      <c r="K115" t="s">
+        <v>16</v>
+      </c>
+      <c r="L115" t="s">
+        <v>16</v>
+      </c>
+      <c r="M115" t="b">
+        <v>0</v>
+      </c>
+      <c r="N115" t="b">
+        <v>1</v>
+      </c>
+      <c r="O115" t="b">
+        <v>0</v>
+      </c>
+      <c r="P115">
+        <v>100</v>
+      </c>
+      <c r="Q115" t="s">
+        <v>20</v>
+      </c>
+      <c r="R115" t="s">
+        <v>21</v>
+      </c>
+      <c r="S115">
+        <f>VLOOKUP($C115,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="T115">
+        <f>VLOOKUP($C115,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>100</v>
+      </c>
+      <c r="U115" t="str">
+        <f>VLOOKUP($C115,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="V115" t="str">
+        <f>VLOOKUP($C115,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>percent</v>
+      </c>
+      <c r="W115" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="116" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A116" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B116" t="s">
+        <v>242</v>
+      </c>
+      <c r="C116" t="s">
+        <v>17</v>
+      </c>
+      <c r="D116" t="s">
+        <v>18</v>
+      </c>
+      <c r="E116" t="s">
+        <v>191</v>
+      </c>
+      <c r="F116" t="s">
+        <v>103</v>
+      </c>
+      <c r="H116" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I116" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J116" t="s">
+        <v>16</v>
+      </c>
+      <c r="K116" t="s">
+        <v>16</v>
+      </c>
+      <c r="L116" t="s">
+        <v>16</v>
+      </c>
+      <c r="M116" t="b">
+        <v>0</v>
+      </c>
+      <c r="N116" t="b">
+        <v>1</v>
+      </c>
+      <c r="O116" t="b">
+        <v>0</v>
+      </c>
+      <c r="P116">
+        <v>100</v>
+      </c>
+      <c r="Q116" t="s">
+        <v>20</v>
+      </c>
+      <c r="R116" t="s">
+        <v>21</v>
+      </c>
+      <c r="S116">
+        <f>VLOOKUP($C116,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-20</v>
+      </c>
+      <c r="T116">
+        <f>VLOOKUP($C116,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="U116" t="str">
+        <f>VLOOKUP($C116,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="V116" t="str">
+        <f>VLOOKUP($C116,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>degree_C</v>
+      </c>
+      <c r="W116" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="117" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A117" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B117" t="s">
+        <v>243</v>
+      </c>
+      <c r="C117" t="s">
+        <v>17</v>
+      </c>
+      <c r="D117" t="s">
+        <v>18</v>
+      </c>
+      <c r="E117" t="s">
+        <v>191</v>
+      </c>
+      <c r="F117" t="s">
+        <v>103</v>
+      </c>
+      <c r="H117" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I117" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J117" t="s">
+        <v>16</v>
+      </c>
+      <c r="K117" t="s">
+        <v>16</v>
+      </c>
+      <c r="L117" t="s">
+        <v>16</v>
+      </c>
+      <c r="M117" t="b">
+        <v>0</v>
+      </c>
+      <c r="N117" t="b">
+        <v>1</v>
+      </c>
+      <c r="O117" t="b">
+        <v>0</v>
+      </c>
+      <c r="P117">
+        <v>100</v>
+      </c>
+      <c r="Q117" t="s">
+        <v>20</v>
+      </c>
+      <c r="R117" t="s">
+        <v>21</v>
+      </c>
+      <c r="S117">
+        <f>VLOOKUP($C117,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-20</v>
+      </c>
+      <c r="T117">
+        <f>VLOOKUP($C117,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="U117" t="str">
+        <f>VLOOKUP($C117,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="V117" t="str">
+        <f>VLOOKUP($C117,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>degree_C</v>
+      </c>
+      <c r="W117" s="2" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="118" spans="1:23" x14ac:dyDescent="0.3">
+      <c r="A118" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B118" t="s">
+        <v>28</v>
+      </c>
+      <c r="C118" t="s">
+        <v>28</v>
+      </c>
+      <c r="D118" t="s">
+        <v>29</v>
+      </c>
+      <c r="E118" t="s">
+        <v>64</v>
+      </c>
+      <c r="F118" t="s">
+        <v>96</v>
+      </c>
+      <c r="H118" s="1">
+        <v>37257</v>
+      </c>
+      <c r="I118" s="1">
+        <v>47484</v>
+      </c>
+      <c r="J118" t="s">
+        <v>16</v>
+      </c>
+      <c r="K118" t="s">
+        <v>16</v>
+      </c>
+      <c r="L118" t="s">
+        <v>16</v>
+      </c>
+      <c r="M118" t="b">
+        <v>0</v>
+      </c>
+      <c r="N118" t="b">
+        <v>1</v>
+      </c>
+      <c r="O118" t="b">
+        <v>0</v>
+      </c>
+      <c r="P118">
+        <v>100</v>
+      </c>
+      <c r="Q118" t="s">
+        <v>20</v>
+      </c>
+      <c r="R118" t="s">
+        <v>21</v>
+      </c>
+      <c r="S118">
+        <f>VLOOKUP($C118,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-10</v>
+      </c>
+      <c r="T118">
+        <f>VLOOKUP($C118,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>10</v>
+      </c>
+      <c r="U118" t="str">
+        <f>VLOOKUP($C118,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="V118" t="str">
+        <f>VLOOKUP($C118,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>m</v>
+      </c>
+      <c r="W118" s="2" t="s">
         <v>232</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add change_naming_convention function and test
</commit_message>
<xml_diff>
--- a/tests/testthat/data-raw/dt_meta.xlsx
+++ b/tests/testthat/data-raw/dt_meta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\plevy\Documents\metamet\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE2265C9-43A6-4054-B5BA-9CFD290FC667}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504630FE-0BFE-418B-BD48-B21DADBDF986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5736" yWindow="324" windowWidth="17280" windowHeight="10596" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
   </bookViews>
@@ -1680,10 +1680,10 @@
   <cols>
     <col min="2" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.77734375" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="0" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="11.21875" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="0" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="26.77734375" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" customWidth="1"/>
+    <col min="8" max="8" width="11.21875" customWidth="1"/>
+    <col min="9" max="9" width="8.88671875" customWidth="1"/>
     <col min="22" max="22" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="26.77734375" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
added edbu data and required changes
</commit_message>
<xml_diff>
--- a/tests/testthat/data-raw/dt_meta.xlsx
+++ b/tests/testthat/data-raw/dt_meta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\plevy\Documents\metamet\data-raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{504630FE-0BFE-418B-BD48-B21DADBDF986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A480153-A5CB-4962-96B3-DA1C3040D664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5736" yWindow="324" windowWidth="17280" windowHeight="10596" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
   </bookViews>
   <sheets>
     <sheet name="dt_meta" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="dt_var_naming" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">dt_meta!$A$1:$X$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">dt_meta!$A$1:$X$119</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1766" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2149" uniqueCount="251">
   <si>
     <t>name_dt</t>
   </si>
@@ -798,7 +798,64 @@
     <t>units_local</t>
   </si>
   <si>
-    <t>TA_2_1_1</t>
+    <t>RH_EB_1_1_1_Avg</t>
+  </si>
+  <si>
+    <t>TA_EB_1_1_1_Avg</t>
+  </si>
+  <si>
+    <t>LWS_EB_7_1_1_Avg</t>
+  </si>
+  <si>
+    <t>PA_EB_1_1_1_Avg</t>
+  </si>
+  <si>
+    <t>P_EB_1_1_1_Tot</t>
+  </si>
+  <si>
+    <t>RN_EB_7_1_1</t>
+  </si>
+  <si>
+    <t>SW_IN_EB_1_1_1</t>
+  </si>
+  <si>
+    <t>PPFD_IN_EB_1_1_1</t>
+  </si>
+  <si>
+    <t>SWC_EB_5_1_1</t>
+  </si>
+  <si>
+    <t>SWC_EB_5_2_1</t>
+  </si>
+  <si>
+    <t>SWC_EB_5_3_1</t>
+  </si>
+  <si>
+    <t>SWC_EB_5_4_1</t>
+  </si>
+  <si>
+    <t>TS_EB_5_1_1</t>
+  </si>
+  <si>
+    <t>TS_EB_5_2_1</t>
+  </si>
+  <si>
+    <t>TS_EB_5_3_1</t>
+  </si>
+  <si>
+    <t>TS_EB_5_4_1</t>
+  </si>
+  <si>
+    <t>G_EB_5_1_1</t>
+  </si>
+  <si>
+    <t>G_EB_5_2_1</t>
+  </si>
+  <si>
+    <t>WTD_EB_5_1_1</t>
+  </si>
+  <si>
+    <t>%Y-%m-%dT%H:%M:%SZ</t>
   </si>
 </sst>
 </file>
@@ -1675,7 +1732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B621CE1-A4D4-4502-917D-92507EE2F7EE}">
-  <dimension ref="A1:X118"/>
+  <dimension ref="A1:X139"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
@@ -1786,7 +1843,9 @@
       <c r="H2" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="I2" s="2"/>
+      <c r="I2" t="s">
+        <v>11</v>
+      </c>
       <c r="J2" t="s">
         <v>11</v>
       </c>
@@ -1862,6 +1921,9 @@
       <c r="H3" t="s">
         <v>90</v>
       </c>
+      <c r="I3" t="s">
+        <v>11</v>
+      </c>
       <c r="J3" t="s">
         <v>11</v>
       </c>
@@ -1940,6 +2002,9 @@
       <c r="H4" t="s">
         <v>90</v>
       </c>
+      <c r="I4" t="s">
+        <v>11</v>
+      </c>
       <c r="J4">
         <v>4</v>
       </c>
@@ -2092,6 +2157,9 @@
       <c r="H6" t="s">
         <v>92</v>
       </c>
+      <c r="I6" t="s">
+        <v>11</v>
+      </c>
       <c r="J6" t="s">
         <v>11</v>
       </c>
@@ -2170,6 +2238,9 @@
       <c r="H7" t="s">
         <v>92</v>
       </c>
+      <c r="I7" t="s">
+        <v>11</v>
+      </c>
       <c r="J7">
         <v>4</v>
       </c>
@@ -2248,6 +2319,9 @@
       <c r="H8" t="s">
         <v>92</v>
       </c>
+      <c r="I8" t="s">
+        <v>11</v>
+      </c>
       <c r="J8">
         <v>4</v>
       </c>
@@ -2326,6 +2400,9 @@
       <c r="H9" t="s">
         <v>93</v>
       </c>
+      <c r="I9" t="s">
+        <v>11</v>
+      </c>
       <c r="J9" t="s">
         <v>11</v>
       </c>
@@ -2404,6 +2481,9 @@
       <c r="H10" t="s">
         <v>93</v>
       </c>
+      <c r="I10" t="s">
+        <v>11</v>
+      </c>
       <c r="J10">
         <v>5</v>
       </c>
@@ -2482,6 +2562,9 @@
       <c r="H11" t="s">
         <v>92</v>
       </c>
+      <c r="I11" t="s">
+        <v>11</v>
+      </c>
       <c r="J11" t="s">
         <v>11</v>
       </c>
@@ -2560,6 +2643,9 @@
       <c r="H12" t="s">
         <v>92</v>
       </c>
+      <c r="I12" t="s">
+        <v>11</v>
+      </c>
       <c r="J12">
         <v>5</v>
       </c>
@@ -2638,6 +2724,9 @@
       <c r="H13" t="s">
         <v>93</v>
       </c>
+      <c r="I13" t="s">
+        <v>11</v>
+      </c>
       <c r="J13">
         <v>4</v>
       </c>
@@ -2716,6 +2805,9 @@
       <c r="H14" t="s">
         <v>93</v>
       </c>
+      <c r="I14" t="s">
+        <v>11</v>
+      </c>
       <c r="J14">
         <v>4</v>
       </c>
@@ -2794,6 +2886,9 @@
       <c r="H15" t="s">
         <v>92</v>
       </c>
+      <c r="I15" t="s">
+        <v>11</v>
+      </c>
       <c r="J15">
         <v>5</v>
       </c>
@@ -2872,6 +2967,9 @@
       <c r="H16" t="s">
         <v>92</v>
       </c>
+      <c r="I16" t="s">
+        <v>11</v>
+      </c>
       <c r="J16">
         <v>5</v>
       </c>
@@ -2950,6 +3048,9 @@
       <c r="H17" t="s">
         <v>92</v>
       </c>
+      <c r="I17" t="s">
+        <v>11</v>
+      </c>
       <c r="J17">
         <v>5</v>
       </c>
@@ -3028,6 +3129,9 @@
       <c r="H18" t="s">
         <v>92</v>
       </c>
+      <c r="I18" t="s">
+        <v>11</v>
+      </c>
       <c r="J18">
         <v>5</v>
       </c>
@@ -3106,6 +3210,9 @@
       <c r="H19" s="2" t="s">
         <v>101</v>
       </c>
+      <c r="I19" t="s">
+        <v>11</v>
+      </c>
       <c r="J19">
         <v>12</v>
       </c>
@@ -3184,6 +3291,9 @@
       <c r="H20" s="2" t="s">
         <v>101</v>
       </c>
+      <c r="I20" t="s">
+        <v>11</v>
+      </c>
       <c r="J20">
         <v>13</v>
       </c>
@@ -3262,6 +3372,9 @@
       <c r="H21" t="s">
         <v>94</v>
       </c>
+      <c r="I21" t="s">
+        <v>11</v>
+      </c>
       <c r="J21">
         <v>4</v>
       </c>
@@ -3340,6 +3453,9 @@
       <c r="H22" t="s">
         <v>92</v>
       </c>
+      <c r="I22" t="s">
+        <v>11</v>
+      </c>
       <c r="J22" t="s">
         <v>11</v>
       </c>
@@ -3418,6 +3534,9 @@
       <c r="H23" t="s">
         <v>92</v>
       </c>
+      <c r="I23" t="s">
+        <v>11</v>
+      </c>
       <c r="J23">
         <v>4</v>
       </c>
@@ -3496,6 +3615,9 @@
       <c r="H24" t="s">
         <v>92</v>
       </c>
+      <c r="I24" t="s">
+        <v>11</v>
+      </c>
       <c r="J24">
         <v>4</v>
       </c>
@@ -3574,6 +3696,9 @@
       <c r="H25" t="s">
         <v>92</v>
       </c>
+      <c r="I25" t="s">
+        <v>11</v>
+      </c>
       <c r="J25">
         <v>5</v>
       </c>
@@ -3652,6 +3777,9 @@
       <c r="H26" t="s">
         <v>92</v>
       </c>
+      <c r="I26" t="s">
+        <v>11</v>
+      </c>
       <c r="J26">
         <v>5</v>
       </c>
@@ -3730,6 +3858,9 @@
       <c r="H27" t="s">
         <v>92</v>
       </c>
+      <c r="I27" t="s">
+        <v>11</v>
+      </c>
       <c r="J27" t="s">
         <v>11</v>
       </c>
@@ -3808,6 +3939,9 @@
       <c r="H28" t="s">
         <v>92</v>
       </c>
+      <c r="I28" t="s">
+        <v>11</v>
+      </c>
       <c r="J28">
         <v>5</v>
       </c>
@@ -3886,6 +4020,9 @@
       <c r="H29" t="s">
         <v>92</v>
       </c>
+      <c r="I29" t="s">
+        <v>11</v>
+      </c>
       <c r="J29">
         <v>4</v>
       </c>
@@ -3964,6 +4101,9 @@
       <c r="H30" t="s">
         <v>95</v>
       </c>
+      <c r="I30" t="s">
+        <v>11</v>
+      </c>
       <c r="J30">
         <v>2</v>
       </c>
@@ -4042,6 +4182,9 @@
       <c r="H31" t="s">
         <v>95</v>
       </c>
+      <c r="I31" t="s">
+        <v>11</v>
+      </c>
       <c r="J31">
         <v>4</v>
       </c>
@@ -4120,6 +4263,9 @@
       <c r="H32" t="s">
         <v>95</v>
       </c>
+      <c r="I32" t="s">
+        <v>11</v>
+      </c>
       <c r="J32">
         <v>7</v>
       </c>
@@ -4198,6 +4344,9 @@
       <c r="H33" t="s">
         <v>92</v>
       </c>
+      <c r="I33" t="s">
+        <v>11</v>
+      </c>
       <c r="J33">
         <v>5</v>
       </c>
@@ -4276,6 +4425,9 @@
       <c r="H34" t="s">
         <v>92</v>
       </c>
+      <c r="I34" t="s">
+        <v>11</v>
+      </c>
       <c r="J34" t="s">
         <v>11</v>
       </c>
@@ -4354,6 +4506,9 @@
       <c r="H35" t="s">
         <v>92</v>
       </c>
+      <c r="I35" t="s">
+        <v>11</v>
+      </c>
       <c r="J35">
         <v>5</v>
       </c>
@@ -4432,6 +4587,9 @@
       <c r="H36" t="s">
         <v>92</v>
       </c>
+      <c r="I36" t="s">
+        <v>11</v>
+      </c>
       <c r="J36">
         <v>7</v>
       </c>
@@ -4510,6 +4668,9 @@
       <c r="H37" t="s">
         <v>92</v>
       </c>
+      <c r="I37" t="s">
+        <v>11</v>
+      </c>
       <c r="J37" t="s">
         <v>11</v>
       </c>
@@ -4588,6 +4749,9 @@
       <c r="H38" t="s">
         <v>92</v>
       </c>
+      <c r="I38" t="s">
+        <v>11</v>
+      </c>
       <c r="J38">
         <v>5</v>
       </c>
@@ -4666,6 +4830,9 @@
       <c r="H39" t="s">
         <v>96</v>
       </c>
+      <c r="I39" t="s">
+        <v>11</v>
+      </c>
       <c r="J39" t="s">
         <v>11</v>
       </c>
@@ -4744,6 +4911,9 @@
       <c r="H40" t="s">
         <v>96</v>
       </c>
+      <c r="I40" t="s">
+        <v>11</v>
+      </c>
       <c r="J40">
         <v>4</v>
       </c>
@@ -4822,6 +4992,9 @@
       <c r="H41" t="s">
         <v>96</v>
       </c>
+      <c r="I41" t="s">
+        <v>11</v>
+      </c>
       <c r="J41">
         <v>4</v>
       </c>
@@ -4900,6 +5073,9 @@
       <c r="H42" t="s">
         <v>96</v>
       </c>
+      <c r="I42" t="s">
+        <v>11</v>
+      </c>
       <c r="J42">
         <v>4</v>
       </c>
@@ -4978,6 +5154,9 @@
       <c r="H43" t="s">
         <v>96</v>
       </c>
+      <c r="I43" t="s">
+        <v>11</v>
+      </c>
       <c r="J43">
         <v>4</v>
       </c>
@@ -5056,6 +5235,9 @@
       <c r="H44" t="s">
         <v>97</v>
       </c>
+      <c r="I44" t="s">
+        <v>11</v>
+      </c>
       <c r="J44">
         <v>2</v>
       </c>
@@ -5134,6 +5316,9 @@
       <c r="H45" t="s">
         <v>97</v>
       </c>
+      <c r="I45" t="s">
+        <v>11</v>
+      </c>
       <c r="J45">
         <v>4</v>
       </c>
@@ -5212,6 +5397,9 @@
       <c r="H46" t="s">
         <v>97</v>
       </c>
+      <c r="I46" t="s">
+        <v>11</v>
+      </c>
       <c r="J46">
         <v>7</v>
       </c>
@@ -5364,6 +5552,9 @@
       <c r="H48" t="s">
         <v>99</v>
       </c>
+      <c r="I48" t="s">
+        <v>11</v>
+      </c>
       <c r="J48">
         <v>6</v>
       </c>
@@ -5442,6 +5633,9 @@
       <c r="H49" s="2" t="s">
         <v>98</v>
       </c>
+      <c r="I49" t="s">
+        <v>11</v>
+      </c>
       <c r="J49">
         <v>6</v>
       </c>
@@ -5520,6 +5714,9 @@
       <c r="H50" t="s">
         <v>99</v>
       </c>
+      <c r="I50" t="s">
+        <v>11</v>
+      </c>
       <c r="J50">
         <v>7</v>
       </c>
@@ -5598,6 +5795,9 @@
       <c r="H51" s="2" t="s">
         <v>98</v>
       </c>
+      <c r="I51" t="s">
+        <v>11</v>
+      </c>
       <c r="J51">
         <v>7</v>
       </c>
@@ -5676,6 +5876,9 @@
       <c r="H52" t="s">
         <v>90</v>
       </c>
+      <c r="I52" t="s">
+        <v>11</v>
+      </c>
       <c r="J52" t="s">
         <v>11</v>
       </c>
@@ -5754,6 +5957,9 @@
       <c r="H53" t="s">
         <v>90</v>
       </c>
+      <c r="I53" t="s">
+        <v>11</v>
+      </c>
       <c r="J53">
         <v>4</v>
       </c>
@@ -5832,6 +6038,9 @@
       <c r="H54" t="s">
         <v>97</v>
       </c>
+      <c r="I54" t="s">
+        <v>11</v>
+      </c>
       <c r="J54" t="s">
         <v>11</v>
       </c>
@@ -5910,6 +6119,9 @@
       <c r="H55" t="s">
         <v>97</v>
       </c>
+      <c r="I55" t="s">
+        <v>11</v>
+      </c>
       <c r="J55">
         <v>4</v>
       </c>
@@ -5988,6 +6200,9 @@
       <c r="H56" t="s">
         <v>97</v>
       </c>
+      <c r="I56" t="s">
+        <v>11</v>
+      </c>
       <c r="J56">
         <v>4</v>
       </c>
@@ -6066,6 +6281,9 @@
       <c r="H57" t="s">
         <v>97</v>
       </c>
+      <c r="I57" t="s">
+        <v>11</v>
+      </c>
       <c r="J57">
         <v>4</v>
       </c>
@@ -6144,6 +6362,9 @@
       <c r="H58" t="s">
         <v>97</v>
       </c>
+      <c r="I58" t="s">
+        <v>11</v>
+      </c>
       <c r="J58">
         <v>4</v>
       </c>
@@ -6222,6 +6443,9 @@
       <c r="H59" t="s">
         <v>97</v>
       </c>
+      <c r="I59" t="s">
+        <v>11</v>
+      </c>
       <c r="J59">
         <v>8</v>
       </c>
@@ -6300,6 +6524,9 @@
       <c r="H60" t="s">
         <v>97</v>
       </c>
+      <c r="I60" t="s">
+        <v>11</v>
+      </c>
       <c r="J60">
         <v>8</v>
       </c>
@@ -6378,6 +6605,9 @@
       <c r="H61" t="s">
         <v>97</v>
       </c>
+      <c r="I61" t="s">
+        <v>11</v>
+      </c>
       <c r="J61">
         <v>8</v>
       </c>
@@ -6456,6 +6686,9 @@
       <c r="H62" t="s">
         <v>97</v>
       </c>
+      <c r="I62" t="s">
+        <v>11</v>
+      </c>
       <c r="J62">
         <v>8</v>
       </c>
@@ -6534,6 +6767,9 @@
       <c r="H63" t="s">
         <v>97</v>
       </c>
+      <c r="I63" t="s">
+        <v>11</v>
+      </c>
       <c r="J63">
         <v>8</v>
       </c>
@@ -6612,6 +6848,9 @@
       <c r="H64" t="s">
         <v>97</v>
       </c>
+      <c r="I64" t="s">
+        <v>11</v>
+      </c>
       <c r="J64">
         <v>9</v>
       </c>
@@ -6690,6 +6929,9 @@
       <c r="H65" t="s">
         <v>97</v>
       </c>
+      <c r="I65" t="s">
+        <v>11</v>
+      </c>
       <c r="J65">
         <v>9</v>
       </c>
@@ -6768,6 +7010,9 @@
       <c r="H66" t="s">
         <v>97</v>
       </c>
+      <c r="I66" t="s">
+        <v>11</v>
+      </c>
       <c r="J66">
         <v>9</v>
       </c>
@@ -6846,6 +7091,9 @@
       <c r="H67" t="s">
         <v>97</v>
       </c>
+      <c r="I67" t="s">
+        <v>11</v>
+      </c>
       <c r="J67">
         <v>9</v>
       </c>
@@ -6924,6 +7172,9 @@
       <c r="H68" t="s">
         <v>97</v>
       </c>
+      <c r="I68" t="s">
+        <v>11</v>
+      </c>
       <c r="J68">
         <v>9</v>
       </c>
@@ -7002,6 +7253,9 @@
       <c r="H69" t="s">
         <v>92</v>
       </c>
+      <c r="I69" t="s">
+        <v>11</v>
+      </c>
       <c r="J69">
         <v>8</v>
       </c>
@@ -7080,6 +7334,9 @@
       <c r="H70" t="s">
         <v>92</v>
       </c>
+      <c r="I70" t="s">
+        <v>11</v>
+      </c>
       <c r="J70">
         <v>9</v>
       </c>
@@ -7158,6 +7415,9 @@
       <c r="H71" t="s">
         <v>92</v>
       </c>
+      <c r="I71" t="s">
+        <v>11</v>
+      </c>
       <c r="J71">
         <v>10</v>
       </c>
@@ -7236,6 +7496,9 @@
       <c r="H72" t="s">
         <v>92</v>
       </c>
+      <c r="I72" t="s">
+        <v>11</v>
+      </c>
       <c r="J72">
         <v>11</v>
       </c>
@@ -7314,6 +7577,9 @@
       <c r="H73" t="s">
         <v>90</v>
       </c>
+      <c r="I73" t="s">
+        <v>11</v>
+      </c>
       <c r="J73">
         <v>8</v>
       </c>
@@ -7392,6 +7658,9 @@
       <c r="H74" t="s">
         <v>90</v>
       </c>
+      <c r="I74" t="s">
+        <v>11</v>
+      </c>
       <c r="J74">
         <v>9</v>
       </c>
@@ -7470,6 +7739,9 @@
       <c r="H75" t="s">
         <v>90</v>
       </c>
+      <c r="I75" t="s">
+        <v>11</v>
+      </c>
       <c r="J75">
         <v>10</v>
       </c>
@@ -7548,6 +7820,9 @@
       <c r="H76" t="s">
         <v>90</v>
       </c>
+      <c r="I76" t="s">
+        <v>11</v>
+      </c>
       <c r="J76">
         <v>11</v>
       </c>
@@ -7626,6 +7901,9 @@
       <c r="H77" t="s">
         <v>96</v>
       </c>
+      <c r="I77" t="s">
+        <v>11</v>
+      </c>
       <c r="J77">
         <v>8</v>
       </c>
@@ -7704,6 +7982,9 @@
       <c r="H78" t="s">
         <v>96</v>
       </c>
+      <c r="I78" t="s">
+        <v>11</v>
+      </c>
       <c r="J78">
         <v>8</v>
       </c>
@@ -7782,6 +8063,9 @@
       <c r="H79" t="s">
         <v>96</v>
       </c>
+      <c r="I79" t="s">
+        <v>11</v>
+      </c>
       <c r="J79">
         <v>8</v>
       </c>
@@ -7860,6 +8144,9 @@
       <c r="H80" t="s">
         <v>96</v>
       </c>
+      <c r="I80" t="s">
+        <v>11</v>
+      </c>
       <c r="J80">
         <v>8</v>
       </c>
@@ -7938,6 +8225,9 @@
       <c r="H81" t="s">
         <v>96</v>
       </c>
+      <c r="I81" t="s">
+        <v>11</v>
+      </c>
       <c r="J81">
         <v>9</v>
       </c>
@@ -8016,6 +8306,9 @@
       <c r="H82" t="s">
         <v>96</v>
       </c>
+      <c r="I82" t="s">
+        <v>11</v>
+      </c>
       <c r="J82">
         <v>9</v>
       </c>
@@ -8094,6 +8387,9 @@
       <c r="H83" t="s">
         <v>96</v>
       </c>
+      <c r="I83" t="s">
+        <v>11</v>
+      </c>
       <c r="J83">
         <v>9</v>
       </c>
@@ -8172,6 +8468,9 @@
       <c r="H84" t="s">
         <v>96</v>
       </c>
+      <c r="I84" t="s">
+        <v>11</v>
+      </c>
       <c r="J84">
         <v>9</v>
       </c>
@@ -8250,6 +8549,9 @@
       <c r="H85" t="s">
         <v>97</v>
       </c>
+      <c r="I85" t="s">
+        <v>11</v>
+      </c>
       <c r="J85">
         <v>10</v>
       </c>
@@ -8328,6 +8630,9 @@
       <c r="H86" t="s">
         <v>97</v>
       </c>
+      <c r="I86" t="s">
+        <v>11</v>
+      </c>
       <c r="J86">
         <v>10</v>
       </c>
@@ -8406,6 +8711,9 @@
       <c r="H87" t="s">
         <v>97</v>
       </c>
+      <c r="I87" t="s">
+        <v>11</v>
+      </c>
       <c r="J87">
         <v>10</v>
       </c>
@@ -8484,6 +8792,9 @@
       <c r="H88" t="s">
         <v>97</v>
       </c>
+      <c r="I88" t="s">
+        <v>11</v>
+      </c>
       <c r="J88">
         <v>10</v>
       </c>
@@ -8562,6 +8873,9 @@
       <c r="H89" t="s">
         <v>97</v>
       </c>
+      <c r="I89" t="s">
+        <v>11</v>
+      </c>
       <c r="J89">
         <v>10</v>
       </c>
@@ -8640,6 +8954,9 @@
       <c r="H90" t="s">
         <v>97</v>
       </c>
+      <c r="I90" t="s">
+        <v>11</v>
+      </c>
       <c r="J90">
         <v>11</v>
       </c>
@@ -8718,6 +9035,9 @@
       <c r="H91" t="s">
         <v>97</v>
       </c>
+      <c r="I91" t="s">
+        <v>11</v>
+      </c>
       <c r="J91">
         <v>11</v>
       </c>
@@ -8796,6 +9116,9 @@
       <c r="H92" t="s">
         <v>97</v>
       </c>
+      <c r="I92" t="s">
+        <v>11</v>
+      </c>
       <c r="J92">
         <v>11</v>
       </c>
@@ -8874,6 +9197,9 @@
       <c r="H93" t="s">
         <v>97</v>
       </c>
+      <c r="I93" t="s">
+        <v>11</v>
+      </c>
       <c r="J93">
         <v>11</v>
       </c>
@@ -8952,6 +9278,9 @@
       <c r="H94" t="s">
         <v>97</v>
       </c>
+      <c r="I94" t="s">
+        <v>11</v>
+      </c>
       <c r="J94">
         <v>11</v>
       </c>
@@ -9030,6 +9359,9 @@
       <c r="H95" t="s">
         <v>96</v>
       </c>
+      <c r="I95" t="s">
+        <v>11</v>
+      </c>
       <c r="J95">
         <v>10</v>
       </c>
@@ -9108,6 +9440,9 @@
       <c r="H96" t="s">
         <v>96</v>
       </c>
+      <c r="I96" t="s">
+        <v>11</v>
+      </c>
       <c r="J96">
         <v>10</v>
       </c>
@@ -9186,6 +9521,9 @@
       <c r="H97" t="s">
         <v>96</v>
       </c>
+      <c r="I97" t="s">
+        <v>11</v>
+      </c>
       <c r="J97">
         <v>10</v>
       </c>
@@ -9264,6 +9602,9 @@
       <c r="H98" t="s">
         <v>96</v>
       </c>
+      <c r="I98" t="s">
+        <v>11</v>
+      </c>
       <c r="J98">
         <v>10</v>
       </c>
@@ -9342,6 +9683,9 @@
       <c r="H99" t="s">
         <v>96</v>
       </c>
+      <c r="I99" t="s">
+        <v>11</v>
+      </c>
       <c r="J99">
         <v>11</v>
       </c>
@@ -9420,6 +9764,9 @@
       <c r="H100" t="s">
         <v>96</v>
       </c>
+      <c r="I100" t="s">
+        <v>11</v>
+      </c>
       <c r="J100">
         <v>11</v>
       </c>
@@ -9498,6 +9845,9 @@
       <c r="H101" t="s">
         <v>96</v>
       </c>
+      <c r="I101" t="s">
+        <v>11</v>
+      </c>
       <c r="J101">
         <v>11</v>
       </c>
@@ -9576,6 +9926,9 @@
       <c r="H102" t="s">
         <v>96</v>
       </c>
+      <c r="I102" t="s">
+        <v>11</v>
+      </c>
       <c r="J102">
         <v>11</v>
       </c>
@@ -9652,6 +10005,9 @@
       <c r="H103" t="s">
         <v>103</v>
       </c>
+      <c r="I103" t="s">
+        <v>11</v>
+      </c>
       <c r="J103" t="s">
         <v>11</v>
       </c>
@@ -9807,6 +10163,9 @@
       <c r="H105" s="2" t="s">
         <v>101</v>
       </c>
+      <c r="I105" t="s">
+        <v>11</v>
+      </c>
       <c r="J105">
         <v>1</v>
       </c>
@@ -9883,6 +10242,9 @@
       <c r="H106" t="s">
         <v>93</v>
       </c>
+      <c r="I106" t="s">
+        <v>11</v>
+      </c>
       <c r="J106">
         <v>1</v>
       </c>
@@ -9959,6 +10321,9 @@
       <c r="H107" t="s">
         <v>97</v>
       </c>
+      <c r="I107" t="s">
+        <v>11</v>
+      </c>
       <c r="J107">
         <v>1</v>
       </c>
@@ -10035,6 +10400,9 @@
       <c r="H108" t="s">
         <v>95</v>
       </c>
+      <c r="I108" t="s">
+        <v>11</v>
+      </c>
       <c r="J108">
         <v>1</v>
       </c>
@@ -10111,6 +10479,9 @@
       <c r="H109" t="s">
         <v>92</v>
       </c>
+      <c r="I109" t="s">
+        <v>11</v>
+      </c>
       <c r="J109">
         <v>1</v>
       </c>
@@ -10187,6 +10558,9 @@
       <c r="H110" t="s">
         <v>92</v>
       </c>
+      <c r="I110" t="s">
+        <v>11</v>
+      </c>
       <c r="J110">
         <v>1</v>
       </c>
@@ -10263,6 +10637,9 @@
       <c r="H111" t="s">
         <v>92</v>
       </c>
+      <c r="I111" t="s">
+        <v>11</v>
+      </c>
       <c r="J111">
         <v>1</v>
       </c>
@@ -10339,6 +10716,9 @@
       <c r="H112" s="2" t="s">
         <v>98</v>
       </c>
+      <c r="I112" t="s">
+        <v>11</v>
+      </c>
       <c r="J112">
         <v>1</v>
       </c>
@@ -10415,6 +10795,9 @@
       <c r="H113" t="s">
         <v>99</v>
       </c>
+      <c r="I113" t="s">
+        <v>11</v>
+      </c>
       <c r="J113">
         <v>1</v>
       </c>
@@ -10491,6 +10874,9 @@
       <c r="H114" t="s">
         <v>96</v>
       </c>
+      <c r="I114" t="s">
+        <v>11</v>
+      </c>
       <c r="J114">
         <v>1</v>
       </c>
@@ -10567,6 +10953,9 @@
       <c r="H115" t="s">
         <v>97</v>
       </c>
+      <c r="I115" t="s">
+        <v>11</v>
+      </c>
       <c r="J115">
         <v>1</v>
       </c>
@@ -10643,6 +11032,9 @@
       <c r="H116" t="s">
         <v>97</v>
       </c>
+      <c r="I116" t="s">
+        <v>11</v>
+      </c>
       <c r="J116">
         <v>1</v>
       </c>
@@ -10719,6 +11111,9 @@
       <c r="H117" t="s">
         <v>90</v>
       </c>
+      <c r="I117" t="s">
+        <v>11</v>
+      </c>
       <c r="J117">
         <v>1</v>
       </c>
@@ -10775,77 +11170,1664 @@
         <v>105</v>
       </c>
       <c r="B118" s="1">
-        <v>34700</v>
+        <v>45139.541666666664</v>
       </c>
       <c r="C118" s="1">
-        <v>47484</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="E118" s="2" t="str">
-        <f>V118&amp;"_"&amp;J118&amp;"_"&amp;K118&amp;"_"&amp;L118</f>
-        <v>TA_2_1_1</v>
+        <v>45292</v>
+      </c>
+      <c r="D118" t="s">
+        <v>103</v>
+      </c>
+      <c r="E118" t="s">
+        <v>103</v>
       </c>
       <c r="F118" t="s">
-        <v>68</v>
+        <v>103</v>
       </c>
       <c r="G118" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="H118" t="s">
-        <v>97</v>
-      </c>
-      <c r="J118">
-        <v>2</v>
-      </c>
-      <c r="K118">
-        <v>1</v>
-      </c>
-      <c r="L118">
-        <v>1</v>
+        <v>103</v>
+      </c>
+      <c r="I118" t="s">
+        <v>11</v>
+      </c>
+      <c r="J118" t="s">
+        <v>11</v>
+      </c>
+      <c r="K118" t="s">
+        <v>11</v>
+      </c>
+      <c r="L118" t="s">
+        <v>11</v>
       </c>
       <c r="M118" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="N118" t="s">
-        <v>16</v>
-      </c>
-      <c r="O118">
+        <v>11</v>
+      </c>
+      <c r="O118" t="e">
         <f>VLOOKUP($V118,naming_lookup!$C$1:$H$40,3,FALSE)</f>
-        <v>-40</v>
-      </c>
-      <c r="P118">
+        <v>#N/A</v>
+      </c>
+      <c r="P118" t="e">
         <f>VLOOKUP($V118,naming_lookup!$C$1:$H$40,4,FALSE)</f>
-        <v>50</v>
-      </c>
-      <c r="Q118">
-        <v>100</v>
-      </c>
-      <c r="R118" s="2" t="s">
-        <v>210</v>
+        <v>#N/A</v>
+      </c>
+      <c r="Q118" t="s">
+        <v>11</v>
+      </c>
+      <c r="R118" t="s">
+        <v>11</v>
       </c>
       <c r="S118" t="str">
         <f>VLOOKUP($V118,naming_lookup!$C$1:$H$40,5,FALSE)</f>
-        <v>t2m</v>
+        <v>site</v>
       </c>
       <c r="T118" t="str">
         <f>VLOOKUP($V118,naming_lookup!$C$1:$H$40,5,FALSE)</f>
-        <v>t2m</v>
+        <v>site</v>
       </c>
       <c r="U118" t="str">
         <f>VLOOKUP($V118,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>NA</v>
+      </c>
+      <c r="V118" t="s">
+        <v>103</v>
+      </c>
+      <c r="W118" t="s">
+        <v>103</v>
+      </c>
+      <c r="X118" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="119" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A119" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B119" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C119" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D119" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E119" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="G119" t="s">
+        <v>11</v>
+      </c>
+      <c r="H119" t="s">
+        <v>91</v>
+      </c>
+      <c r="I119" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="J119" t="s">
+        <v>11</v>
+      </c>
+      <c r="K119" t="s">
+        <v>11</v>
+      </c>
+      <c r="L119" t="s">
+        <v>11</v>
+      </c>
+      <c r="M119" t="s">
+        <v>15</v>
+      </c>
+      <c r="N119" t="s">
+        <v>16</v>
+      </c>
+      <c r="O119" t="e">
+        <f>VLOOKUP($V119,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="P119" t="e">
+        <f>VLOOKUP($V119,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>#N/A</v>
+      </c>
+      <c r="Q119" t="s">
+        <v>11</v>
+      </c>
+      <c r="R119" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="S119" t="str">
+        <f>VLOOKUP($V119,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>time</v>
+      </c>
+      <c r="T119" t="str">
+        <f>VLOOKUP($V119,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>time</v>
+      </c>
+      <c r="U119" t="str">
+        <f>VLOOKUP($V119,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>NA</v>
+      </c>
+      <c r="V119" t="s">
+        <v>85</v>
+      </c>
+      <c r="W119" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="X119" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="120" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A120" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B120" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C120" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D120" t="s">
+        <v>231</v>
+      </c>
+      <c r="E120" t="s">
+        <v>231</v>
+      </c>
+      <c r="F120" t="s">
+        <v>70</v>
+      </c>
+      <c r="G120" t="s">
+        <v>158</v>
+      </c>
+      <c r="H120" t="s">
+        <v>95</v>
+      </c>
+      <c r="I120" t="s">
+        <v>11</v>
+      </c>
+      <c r="J120">
+        <v>1</v>
+      </c>
+      <c r="K120">
+        <v>1</v>
+      </c>
+      <c r="L120">
+        <v>1</v>
+      </c>
+      <c r="M120" t="s">
+        <v>15</v>
+      </c>
+      <c r="N120" t="s">
+        <v>16</v>
+      </c>
+      <c r="O120">
+        <f>VLOOKUP($V120,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>30</v>
+      </c>
+      <c r="P120">
+        <f>VLOOKUP($V120,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>120</v>
+      </c>
+      <c r="Q120">
+        <v>100</v>
+      </c>
+      <c r="R120" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S120" t="str">
+        <f>VLOOKUP($V120,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>rh</v>
+      </c>
+      <c r="T120" t="str">
+        <f>VLOOKUP($V120,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>rh</v>
+      </c>
+      <c r="U120" t="str">
+        <f>VLOOKUP($V120,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>percent</v>
+      </c>
+      <c r="V120" t="s">
+        <v>69</v>
+      </c>
+      <c r="W120" t="s">
+        <v>70</v>
+      </c>
+      <c r="X120" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="121" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A121" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B121" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C121" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D121" t="s">
+        <v>232</v>
+      </c>
+      <c r="E121" t="s">
+        <v>232</v>
+      </c>
+      <c r="F121" t="s">
+        <v>68</v>
+      </c>
+      <c r="G121" t="s">
+        <v>174</v>
+      </c>
+      <c r="H121" t="s">
+        <v>97</v>
+      </c>
+      <c r="I121" t="s">
+        <v>11</v>
+      </c>
+      <c r="J121">
+        <v>1</v>
+      </c>
+      <c r="K121">
+        <v>1</v>
+      </c>
+      <c r="L121">
+        <v>1</v>
+      </c>
+      <c r="M121" t="s">
+        <v>15</v>
+      </c>
+      <c r="N121" t="s">
+        <v>16</v>
+      </c>
+      <c r="O121">
+        <f>VLOOKUP($V121,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-40</v>
+      </c>
+      <c r="P121">
+        <f>VLOOKUP($V121,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="Q121">
+        <v>100</v>
+      </c>
+      <c r="R121" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S121" t="str">
+        <f>VLOOKUP($V121,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>t2m</v>
+      </c>
+      <c r="T121" t="str">
+        <f>VLOOKUP($V121,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>t2m</v>
+      </c>
+      <c r="U121" t="str">
+        <f>VLOOKUP($V121,naming_lookup!$C$1:$H$40,6,FALSE)</f>
         <v>degree_C</v>
       </c>
-      <c r="V118" t="s">
+      <c r="V121" t="s">
         <v>67</v>
       </c>
-      <c r="W118" t="s">
+      <c r="W121" t="s">
         <v>68</v>
       </c>
-      <c r="X118" t="s">
-        <v>14</v>
-      </c>
+      <c r="X121" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="122" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A122" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B122" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C122" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D122" t="s">
+        <v>233</v>
+      </c>
+      <c r="E122" t="s">
+        <v>233</v>
+      </c>
+      <c r="F122" t="s">
+        <v>82</v>
+      </c>
+      <c r="G122" t="s">
+        <v>83</v>
+      </c>
+      <c r="H122" t="s">
+        <v>93</v>
+      </c>
+      <c r="I122" t="s">
+        <v>11</v>
+      </c>
+      <c r="J122">
+        <v>7</v>
+      </c>
+      <c r="K122">
+        <v>1</v>
+      </c>
+      <c r="L122">
+        <v>1</v>
+      </c>
+      <c r="M122" t="s">
+        <v>15</v>
+      </c>
+      <c r="N122" t="s">
+        <v>16</v>
+      </c>
+      <c r="O122">
+        <f>VLOOKUP($V122,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-99999</v>
+      </c>
+      <c r="P122">
+        <f>VLOOKUP($V122,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>99999</v>
+      </c>
+      <c r="Q122">
+        <v>100</v>
+      </c>
+      <c r="R122" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S122" t="str">
+        <f>VLOOKUP($V122,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>rh</v>
+      </c>
+      <c r="T122" t="str">
+        <f>VLOOKUP($V122,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>rh</v>
+      </c>
+      <c r="U122">
+        <f>VLOOKUP($V122,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>1</v>
+      </c>
+      <c r="V122" t="s">
+        <v>135</v>
+      </c>
+      <c r="W122" t="s">
+        <v>82</v>
+      </c>
+      <c r="X122" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="123" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A123" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B123" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C123" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D123" t="s">
+        <v>234</v>
+      </c>
+      <c r="E123" t="s">
+        <v>234</v>
+      </c>
+      <c r="F123" t="s">
+        <v>29</v>
+      </c>
+      <c r="G123" t="s">
+        <v>30</v>
+      </c>
+      <c r="H123" t="s">
+        <v>94</v>
+      </c>
+      <c r="I123" t="s">
+        <v>11</v>
+      </c>
+      <c r="J123">
+        <v>1</v>
+      </c>
+      <c r="K123">
+        <v>1</v>
+      </c>
+      <c r="L123">
+        <v>1</v>
+      </c>
+      <c r="M123" t="s">
+        <v>15</v>
+      </c>
+      <c r="N123" t="s">
+        <v>16</v>
+      </c>
+      <c r="O123">
+        <f>VLOOKUP($V123,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>90</v>
+      </c>
+      <c r="P123">
+        <f>VLOOKUP($V123,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>130</v>
+      </c>
+      <c r="Q123">
+        <v>100</v>
+      </c>
+      <c r="R123" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S123" t="str">
+        <f>VLOOKUP($V123,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>sp</v>
+      </c>
+      <c r="T123" t="str">
+        <f>VLOOKUP($V123,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>sp</v>
+      </c>
+      <c r="U123" t="str">
+        <f>VLOOKUP($V123,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>kPa</v>
+      </c>
+      <c r="V123" t="s">
+        <v>28</v>
+      </c>
+      <c r="W123" t="s">
+        <v>29</v>
+      </c>
+      <c r="X123" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="124" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A124" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B124" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C124" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D124" t="s">
+        <v>235</v>
+      </c>
+      <c r="E124" t="s">
+        <v>235</v>
+      </c>
+      <c r="F124" t="s">
+        <v>49</v>
+      </c>
+      <c r="G124" t="s">
+        <v>208</v>
+      </c>
+      <c r="H124" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="I124" t="s">
+        <v>11</v>
+      </c>
+      <c r="J124">
+        <v>1</v>
+      </c>
+      <c r="K124">
+        <v>1</v>
+      </c>
+      <c r="L124">
+        <v>1</v>
+      </c>
+      <c r="M124" t="s">
+        <v>15</v>
+      </c>
+      <c r="N124" t="s">
+        <v>16</v>
+      </c>
+      <c r="O124">
+        <f>VLOOKUP($V124,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="P124">
+        <f>VLOOKUP($V124,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="Q124">
+        <v>100</v>
+      </c>
+      <c r="R124" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S124" t="str">
+        <f>VLOOKUP($V124,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>tp</v>
+      </c>
+      <c r="T124" t="str">
+        <f>VLOOKUP($V124,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>tp</v>
+      </c>
+      <c r="U124" t="str">
+        <f>VLOOKUP($V124,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>mm</v>
+      </c>
+      <c r="V124" t="s">
+        <v>48</v>
+      </c>
+      <c r="W124" t="s">
+        <v>49</v>
+      </c>
+      <c r="X124" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="125" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A125" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B125" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C125" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D125" t="s">
+        <v>236</v>
+      </c>
+      <c r="E125" t="s">
+        <v>236</v>
+      </c>
+      <c r="F125" t="s">
+        <v>60</v>
+      </c>
+      <c r="G125" t="s">
+        <v>125</v>
+      </c>
+      <c r="H125" t="s">
+        <v>92</v>
+      </c>
+      <c r="I125" t="s">
+        <v>11</v>
+      </c>
+      <c r="J125">
+        <v>7</v>
+      </c>
+      <c r="K125">
+        <v>1</v>
+      </c>
+      <c r="L125">
+        <v>1</v>
+      </c>
+      <c r="M125" t="s">
+        <v>15</v>
+      </c>
+      <c r="N125" t="s">
+        <v>16</v>
+      </c>
+      <c r="O125">
+        <f>VLOOKUP($V125,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-500</v>
+      </c>
+      <c r="P125">
+        <f>VLOOKUP($V125,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>1200</v>
+      </c>
+      <c r="Q125">
+        <v>100</v>
+      </c>
+      <c r="R125" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S125" t="str">
+        <f>VLOOKUP($V125,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>rn</v>
+      </c>
+      <c r="T125" t="str">
+        <f>VLOOKUP($V125,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>rn</v>
+      </c>
+      <c r="U125" t="str">
+        <f>VLOOKUP($V125,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>W / m^2</v>
+      </c>
+      <c r="V125" t="s">
+        <v>100</v>
+      </c>
+      <c r="W125" t="s">
+        <v>60</v>
+      </c>
+      <c r="X125" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="126" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A126" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B126" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C126" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D126" t="s">
+        <v>237</v>
+      </c>
+      <c r="E126" t="s">
+        <v>237</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="G126" t="s">
+        <v>125</v>
+      </c>
+      <c r="H126" t="s">
+        <v>92</v>
+      </c>
+      <c r="I126" t="s">
+        <v>11</v>
+      </c>
+      <c r="J126">
+        <v>1</v>
+      </c>
+      <c r="K126">
+        <v>1</v>
+      </c>
+      <c r="L126">
+        <v>1</v>
+      </c>
+      <c r="M126" t="s">
+        <v>15</v>
+      </c>
+      <c r="N126" t="s">
+        <v>16</v>
+      </c>
+      <c r="O126">
+        <f>VLOOKUP($V126,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="P126">
+        <f>VLOOKUP($V126,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>1200</v>
+      </c>
+      <c r="Q126">
+        <v>100</v>
+      </c>
+      <c r="R126" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S126" t="str">
+        <f>VLOOKUP($V126,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="T126" t="str">
+        <f>VLOOKUP($V126,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="U126" t="str">
+        <f>VLOOKUP($V126,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>W / m^2</v>
+      </c>
+      <c r="V126" t="s">
+        <v>31</v>
+      </c>
+      <c r="W126" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="X126" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A127" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B127" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C127" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D127" t="s">
+        <v>238</v>
+      </c>
+      <c r="E127" t="s">
+        <v>238</v>
+      </c>
+      <c r="F127" t="s">
+        <v>41</v>
+      </c>
+      <c r="G127" t="s">
+        <v>138</v>
+      </c>
+      <c r="H127" t="s">
+        <v>92</v>
+      </c>
+      <c r="I127" t="s">
+        <v>11</v>
+      </c>
+      <c r="J127">
+        <v>1</v>
+      </c>
+      <c r="K127">
+        <v>1</v>
+      </c>
+      <c r="L127">
+        <v>1</v>
+      </c>
+      <c r="M127" t="s">
+        <v>15</v>
+      </c>
+      <c r="N127" t="s">
+        <v>16</v>
+      </c>
+      <c r="O127">
+        <f>VLOOKUP($V127,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="P127">
+        <f>VLOOKUP($V127,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>2200</v>
+      </c>
+      <c r="Q127">
+        <v>100</v>
+      </c>
+      <c r="R127" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S127" t="str">
+        <f>VLOOKUP($V127,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="T127" t="str">
+        <f>VLOOKUP($V127,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="U127" t="str">
+        <f>VLOOKUP($V127,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>micromol / m^2 / s</v>
+      </c>
+      <c r="V127" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="W127" t="s">
+        <v>41</v>
+      </c>
+      <c r="X127" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="128" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A128" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B128" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C128" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D128" t="s">
+        <v>239</v>
+      </c>
+      <c r="E128" t="s">
+        <v>239</v>
+      </c>
+      <c r="F128" t="s">
+        <v>18</v>
+      </c>
+      <c r="G128" t="s">
+        <v>158</v>
+      </c>
+      <c r="H128" t="s">
+        <v>96</v>
+      </c>
+      <c r="I128" t="s">
+        <v>11</v>
+      </c>
+      <c r="J128">
+        <v>5</v>
+      </c>
+      <c r="K128">
+        <v>1</v>
+      </c>
+      <c r="L128">
+        <v>1</v>
+      </c>
+      <c r="M128" t="s">
+        <v>15</v>
+      </c>
+      <c r="N128" t="s">
+        <v>16</v>
+      </c>
+      <c r="O128">
+        <f>VLOOKUP($V128,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="P128">
+        <f>VLOOKUP($V128,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>100</v>
+      </c>
+      <c r="Q128">
+        <v>100</v>
+      </c>
+      <c r="R128" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S128" t="str">
+        <f>VLOOKUP($V128,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="T128" t="str">
+        <f>VLOOKUP($V128,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="U128" t="str">
+        <f>VLOOKUP($V128,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>percent</v>
+      </c>
+      <c r="V128" t="s">
+        <v>17</v>
+      </c>
+      <c r="W128" t="s">
+        <v>18</v>
+      </c>
+      <c r="X128" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="129" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A129" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B129" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C129" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D129" t="s">
+        <v>240</v>
+      </c>
+      <c r="E129" t="s">
+        <v>240</v>
+      </c>
+      <c r="F129" t="s">
+        <v>18</v>
+      </c>
+      <c r="G129" t="s">
+        <v>158</v>
+      </c>
+      <c r="H129" t="s">
+        <v>96</v>
+      </c>
+      <c r="I129" t="s">
+        <v>11</v>
+      </c>
+      <c r="J129">
+        <v>5</v>
+      </c>
+      <c r="K129">
+        <v>2</v>
+      </c>
+      <c r="L129">
+        <v>1</v>
+      </c>
+      <c r="M129" t="s">
+        <v>15</v>
+      </c>
+      <c r="N129" t="s">
+        <v>16</v>
+      </c>
+      <c r="O129">
+        <f>VLOOKUP($V129,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="P129">
+        <f>VLOOKUP($V129,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>100</v>
+      </c>
+      <c r="Q129">
+        <v>100</v>
+      </c>
+      <c r="R129" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S129" t="str">
+        <f>VLOOKUP($V129,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="T129" t="str">
+        <f>VLOOKUP($V129,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="U129" t="str">
+        <f>VLOOKUP($V129,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>percent</v>
+      </c>
+      <c r="V129" t="s">
+        <v>17</v>
+      </c>
+      <c r="W129" t="s">
+        <v>18</v>
+      </c>
+      <c r="X129" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="130" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A130" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B130" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C130" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D130" t="s">
+        <v>241</v>
+      </c>
+      <c r="E130" t="s">
+        <v>241</v>
+      </c>
+      <c r="F130" t="s">
+        <v>18</v>
+      </c>
+      <c r="G130" t="s">
+        <v>158</v>
+      </c>
+      <c r="H130" t="s">
+        <v>96</v>
+      </c>
+      <c r="I130" t="s">
+        <v>11</v>
+      </c>
+      <c r="J130">
+        <v>5</v>
+      </c>
+      <c r="K130">
+        <v>3</v>
+      </c>
+      <c r="L130">
+        <v>1</v>
+      </c>
+      <c r="M130" t="s">
+        <v>15</v>
+      </c>
+      <c r="N130" t="s">
+        <v>16</v>
+      </c>
+      <c r="O130">
+        <f>VLOOKUP($V130,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="P130">
+        <f>VLOOKUP($V130,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>100</v>
+      </c>
+      <c r="Q130">
+        <v>100</v>
+      </c>
+      <c r="R130" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S130" t="str">
+        <f>VLOOKUP($V130,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="T130" t="str">
+        <f>VLOOKUP($V130,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="U130" t="str">
+        <f>VLOOKUP($V130,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>percent</v>
+      </c>
+      <c r="V130" t="s">
+        <v>17</v>
+      </c>
+      <c r="W130" t="s">
+        <v>18</v>
+      </c>
+      <c r="X130" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="131" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A131" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B131" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C131" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D131" t="s">
+        <v>242</v>
+      </c>
+      <c r="E131" t="s">
+        <v>242</v>
+      </c>
+      <c r="F131" t="s">
+        <v>18</v>
+      </c>
+      <c r="G131" t="s">
+        <v>158</v>
+      </c>
+      <c r="H131" t="s">
+        <v>96</v>
+      </c>
+      <c r="I131" t="s">
+        <v>11</v>
+      </c>
+      <c r="J131">
+        <v>5</v>
+      </c>
+      <c r="K131">
+        <v>4</v>
+      </c>
+      <c r="L131">
+        <v>1</v>
+      </c>
+      <c r="M131" t="s">
+        <v>15</v>
+      </c>
+      <c r="N131" t="s">
+        <v>16</v>
+      </c>
+      <c r="O131">
+        <f>VLOOKUP($V131,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>0</v>
+      </c>
+      <c r="P131">
+        <f>VLOOKUP($V131,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>100</v>
+      </c>
+      <c r="Q131">
+        <v>100</v>
+      </c>
+      <c r="R131" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S131" t="str">
+        <f>VLOOKUP($V131,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="T131" t="str">
+        <f>VLOOKUP($V131,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="U131" t="str">
+        <f>VLOOKUP($V131,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>percent</v>
+      </c>
+      <c r="V131" t="s">
+        <v>17</v>
+      </c>
+      <c r="W131" t="s">
+        <v>18</v>
+      </c>
+      <c r="X131" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="132" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A132" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B132" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C132" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D132" t="s">
+        <v>243</v>
+      </c>
+      <c r="E132" t="s">
+        <v>243</v>
+      </c>
+      <c r="F132" t="s">
+        <v>13</v>
+      </c>
+      <c r="G132" t="s">
+        <v>174</v>
+      </c>
+      <c r="H132" t="s">
+        <v>97</v>
+      </c>
+      <c r="I132" t="s">
+        <v>11</v>
+      </c>
+      <c r="J132">
+        <v>5</v>
+      </c>
+      <c r="K132">
+        <v>1</v>
+      </c>
+      <c r="L132">
+        <v>1</v>
+      </c>
+      <c r="M132" t="s">
+        <v>15</v>
+      </c>
+      <c r="N132" t="s">
+        <v>16</v>
+      </c>
+      <c r="O132">
+        <f>VLOOKUP($V132,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-20</v>
+      </c>
+      <c r="P132">
+        <f>VLOOKUP($V132,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="Q132">
+        <v>100</v>
+      </c>
+      <c r="R132" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S132" t="str">
+        <f>VLOOKUP($V132,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="T132" t="str">
+        <f>VLOOKUP($V132,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="U132" t="str">
+        <f>VLOOKUP($V132,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>degree_C</v>
+      </c>
+      <c r="V132" t="s">
+        <v>12</v>
+      </c>
+      <c r="W132" t="s">
+        <v>13</v>
+      </c>
+      <c r="X132" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="133" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A133" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B133" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C133" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D133" t="s">
+        <v>244</v>
+      </c>
+      <c r="E133" t="s">
+        <v>244</v>
+      </c>
+      <c r="F133" t="s">
+        <v>13</v>
+      </c>
+      <c r="G133" t="s">
+        <v>174</v>
+      </c>
+      <c r="H133" t="s">
+        <v>97</v>
+      </c>
+      <c r="I133" t="s">
+        <v>11</v>
+      </c>
+      <c r="J133">
+        <v>5</v>
+      </c>
+      <c r="K133">
+        <v>2</v>
+      </c>
+      <c r="L133">
+        <v>1</v>
+      </c>
+      <c r="M133" t="s">
+        <v>15</v>
+      </c>
+      <c r="N133" t="s">
+        <v>16</v>
+      </c>
+      <c r="O133">
+        <f>VLOOKUP($V133,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-20</v>
+      </c>
+      <c r="P133">
+        <f>VLOOKUP($V133,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="Q133">
+        <v>100</v>
+      </c>
+      <c r="R133" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S133" t="str">
+        <f>VLOOKUP($V133,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="T133" t="str">
+        <f>VLOOKUP($V133,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="U133" t="str">
+        <f>VLOOKUP($V133,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>degree_C</v>
+      </c>
+      <c r="V133" t="s">
+        <v>12</v>
+      </c>
+      <c r="W133" t="s">
+        <v>13</v>
+      </c>
+      <c r="X133" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="134" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A134" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B134" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C134" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D134" t="s">
+        <v>245</v>
+      </c>
+      <c r="E134" t="s">
+        <v>245</v>
+      </c>
+      <c r="F134" t="s">
+        <v>13</v>
+      </c>
+      <c r="G134" t="s">
+        <v>174</v>
+      </c>
+      <c r="H134" t="s">
+        <v>97</v>
+      </c>
+      <c r="I134" t="s">
+        <v>11</v>
+      </c>
+      <c r="J134">
+        <v>5</v>
+      </c>
+      <c r="K134">
+        <v>3</v>
+      </c>
+      <c r="L134">
+        <v>1</v>
+      </c>
+      <c r="M134" t="s">
+        <v>15</v>
+      </c>
+      <c r="N134" t="s">
+        <v>16</v>
+      </c>
+      <c r="O134">
+        <f>VLOOKUP($V134,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-20</v>
+      </c>
+      <c r="P134">
+        <f>VLOOKUP($V134,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="Q134">
+        <v>100</v>
+      </c>
+      <c r="R134" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S134" t="str">
+        <f>VLOOKUP($V134,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="T134" t="str">
+        <f>VLOOKUP($V134,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="U134" t="str">
+        <f>VLOOKUP($V134,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>degree_C</v>
+      </c>
+      <c r="V134" t="s">
+        <v>12</v>
+      </c>
+      <c r="W134" t="s">
+        <v>13</v>
+      </c>
+      <c r="X134" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="135" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A135" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B135" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C135" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D135" t="s">
+        <v>246</v>
+      </c>
+      <c r="E135" t="s">
+        <v>246</v>
+      </c>
+      <c r="F135" t="s">
+        <v>13</v>
+      </c>
+      <c r="G135" t="s">
+        <v>174</v>
+      </c>
+      <c r="H135" t="s">
+        <v>97</v>
+      </c>
+      <c r="I135" t="s">
+        <v>11</v>
+      </c>
+      <c r="J135">
+        <v>5</v>
+      </c>
+      <c r="K135">
+        <v>4</v>
+      </c>
+      <c r="L135">
+        <v>1</v>
+      </c>
+      <c r="M135" t="s">
+        <v>15</v>
+      </c>
+      <c r="N135" t="s">
+        <v>16</v>
+      </c>
+      <c r="O135">
+        <f>VLOOKUP($V135,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-20</v>
+      </c>
+      <c r="P135">
+        <f>VLOOKUP($V135,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>50</v>
+      </c>
+      <c r="Q135">
+        <v>100</v>
+      </c>
+      <c r="R135" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S135" t="str">
+        <f>VLOOKUP($V135,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="T135" t="str">
+        <f>VLOOKUP($V135,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>stl1</v>
+      </c>
+      <c r="U135" t="str">
+        <f>VLOOKUP($V135,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>degree_C</v>
+      </c>
+      <c r="V135" t="s">
+        <v>12</v>
+      </c>
+      <c r="W135" t="s">
+        <v>13</v>
+      </c>
+      <c r="X135" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="136" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A136" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B136" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C136" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D136" t="s">
+        <v>247</v>
+      </c>
+      <c r="E136" t="s">
+        <v>247</v>
+      </c>
+      <c r="F136" t="s">
+        <v>21</v>
+      </c>
+      <c r="G136" t="s">
+        <v>22</v>
+      </c>
+      <c r="H136" t="s">
+        <v>92</v>
+      </c>
+      <c r="I136" t="s">
+        <v>11</v>
+      </c>
+      <c r="J136">
+        <v>5</v>
+      </c>
+      <c r="K136">
+        <v>1</v>
+      </c>
+      <c r="L136">
+        <v>1</v>
+      </c>
+      <c r="M136" t="s">
+        <v>15</v>
+      </c>
+      <c r="N136" t="s">
+        <v>16</v>
+      </c>
+      <c r="O136">
+        <f>VLOOKUP($V136,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-30</v>
+      </c>
+      <c r="P136">
+        <f>VLOOKUP($V136,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>30</v>
+      </c>
+      <c r="Q136">
+        <v>100</v>
+      </c>
+      <c r="R136" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S136" t="str">
+        <f>VLOOKUP($V136,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="T136" t="str">
+        <f>VLOOKUP($V136,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="U136" t="str">
+        <f>VLOOKUP($V136,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>W / m^2</v>
+      </c>
+      <c r="V136" t="s">
+        <v>20</v>
+      </c>
+      <c r="W136" t="s">
+        <v>21</v>
+      </c>
+      <c r="X136" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="137" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A137" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B137" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C137" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D137" t="s">
+        <v>248</v>
+      </c>
+      <c r="E137" t="s">
+        <v>248</v>
+      </c>
+      <c r="F137" t="s">
+        <v>21</v>
+      </c>
+      <c r="G137" t="s">
+        <v>22</v>
+      </c>
+      <c r="H137" t="s">
+        <v>92</v>
+      </c>
+      <c r="I137" t="s">
+        <v>11</v>
+      </c>
+      <c r="J137">
+        <v>5</v>
+      </c>
+      <c r="K137">
+        <v>2</v>
+      </c>
+      <c r="L137">
+        <v>1</v>
+      </c>
+      <c r="M137" t="s">
+        <v>15</v>
+      </c>
+      <c r="N137" t="s">
+        <v>16</v>
+      </c>
+      <c r="O137">
+        <f>VLOOKUP($V137,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-30</v>
+      </c>
+      <c r="P137">
+        <f>VLOOKUP($V137,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>30</v>
+      </c>
+      <c r="Q137">
+        <v>100</v>
+      </c>
+      <c r="R137" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S137" t="str">
+        <f>VLOOKUP($V137,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="T137" t="str">
+        <f>VLOOKUP($V137,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>ssrd</v>
+      </c>
+      <c r="U137" t="str">
+        <f>VLOOKUP($V137,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>W / m^2</v>
+      </c>
+      <c r="V137" t="s">
+        <v>20</v>
+      </c>
+      <c r="W137" t="s">
+        <v>21</v>
+      </c>
+      <c r="X137" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="138" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A138" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B138" s="1">
+        <v>45139.541666666664</v>
+      </c>
+      <c r="C138" s="1">
+        <v>45292</v>
+      </c>
+      <c r="D138" t="s">
+        <v>249</v>
+      </c>
+      <c r="E138" t="s">
+        <v>249</v>
+      </c>
+      <c r="F138" t="s">
+        <v>24</v>
+      </c>
+      <c r="G138" t="s">
+        <v>59</v>
+      </c>
+      <c r="H138" t="s">
+        <v>90</v>
+      </c>
+      <c r="I138" t="s">
+        <v>11</v>
+      </c>
+      <c r="J138">
+        <v>5</v>
+      </c>
+      <c r="K138">
+        <v>1</v>
+      </c>
+      <c r="L138">
+        <v>1</v>
+      </c>
+      <c r="M138" t="s">
+        <v>15</v>
+      </c>
+      <c r="N138" t="s">
+        <v>16</v>
+      </c>
+      <c r="O138">
+        <f>VLOOKUP($V138,naming_lookup!$C$1:$H$40,3,FALSE)</f>
+        <v>-10</v>
+      </c>
+      <c r="P138">
+        <f>VLOOKUP($V138,naming_lookup!$C$1:$H$40,4,FALSE)</f>
+        <v>10</v>
+      </c>
+      <c r="Q138">
+        <v>100</v>
+      </c>
+      <c r="R138" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="S138" t="str">
+        <f>VLOOKUP($V138,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="T138" t="str">
+        <f>VLOOKUP($V138,naming_lookup!$C$1:$H$40,5,FALSE)</f>
+        <v>swvl1</v>
+      </c>
+      <c r="U138" t="str">
+        <f>VLOOKUP($V138,naming_lookup!$C$1:$H$40,6,FALSE)</f>
+        <v>m</v>
+      </c>
+      <c r="V138" t="s">
+        <v>23</v>
+      </c>
+      <c r="W138" t="s">
+        <v>24</v>
+      </c>
+      <c r="X138" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="139" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A139" s="2"/>
+      <c r="B139" s="1"/>
+      <c r="C139" s="1"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E3:N53">

</xml_diff>

<commit_message>
27/03/2026, CC: created upload raw data tab and metamet obj creation
</commit_message>
<xml_diff>
--- a/tests/testthat/data-raw/dt_meta.xlsx
+++ b/tests/testthat/data-raw/dt_meta.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\plevy\Documents\metamet\data-raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cehacuk-my.sharepoint.com/personal/clacap_ceh_ac_uk/Documents/metamet/tests/testthat/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A480153-A5CB-4962-96B3-DA1C3040D664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{3A480153-A5CB-4962-96B3-DA1C3040D664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA9B4E97-8CB5-4EF9-BF9B-68D61D592B8D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
   </bookViews>
   <sheets>
     <sheet name="dt_meta" sheetId="1" r:id="rId1"/>
@@ -1733,19 +1733,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B621CE1-A4D4-4502-917D-92507EE2F7EE}">
   <dimension ref="A1:X139"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="3" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26.77734375" customWidth="1"/>
-    <col min="7" max="7" width="8.88671875" customWidth="1"/>
-    <col min="8" max="8" width="11.21875" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" customWidth="1"/>
-    <col min="22" max="22" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="26.77734375" customWidth="1"/>
+    <col min="2" max="3" width="15.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="17.90625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.81640625" customWidth="1"/>
+    <col min="7" max="7" width="8.90625" customWidth="1"/>
+    <col min="8" max="8" width="11.1796875" customWidth="1"/>
+    <col min="9" max="9" width="8.90625" customWidth="1"/>
+    <col min="17" max="17" width="10.1796875" customWidth="1"/>
+    <col min="22" max="22" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="26.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>103</v>
       </c>
@@ -1819,7 +1820,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>104</v>
       </c>
@@ -1894,7 +1895,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>104</v>
       </c>
@@ -1975,7 +1976,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>104</v>
       </c>
@@ -2056,7 +2057,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>104</v>
       </c>
@@ -2130,7 +2131,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>104</v>
       </c>
@@ -2211,7 +2212,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>104</v>
       </c>
@@ -2292,7 +2293,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>104</v>
       </c>
@@ -2373,7 +2374,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>104</v>
       </c>
@@ -2454,7 +2455,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>104</v>
       </c>
@@ -2535,7 +2536,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>104</v>
       </c>
@@ -2616,7 +2617,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>104</v>
       </c>
@@ -2697,7 +2698,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>104</v>
       </c>
@@ -2778,7 +2779,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>104</v>
       </c>
@@ -2859,7 +2860,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>104</v>
       </c>
@@ -2940,7 +2941,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>104</v>
       </c>
@@ -3021,7 +3022,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>104</v>
       </c>
@@ -3102,7 +3103,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>104</v>
       </c>
@@ -3183,7 +3184,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>104</v>
       </c>
@@ -3264,7 +3265,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="20" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>104</v>
       </c>
@@ -3345,7 +3346,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="21" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>104</v>
       </c>
@@ -3426,7 +3427,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>104</v>
       </c>
@@ -3507,7 +3508,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>104</v>
       </c>
@@ -3588,7 +3589,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>104</v>
       </c>
@@ -3669,7 +3670,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>104</v>
       </c>
@@ -3750,7 +3751,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>104</v>
       </c>
@@ -3831,7 +3832,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>104</v>
       </c>
@@ -3912,7 +3913,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>104</v>
       </c>
@@ -3993,7 +3994,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>104</v>
       </c>
@@ -4074,7 +4075,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>104</v>
       </c>
@@ -4155,7 +4156,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>104</v>
       </c>
@@ -4236,7 +4237,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>104</v>
       </c>
@@ -4317,7 +4318,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>104</v>
       </c>
@@ -4398,7 +4399,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>104</v>
       </c>
@@ -4479,7 +4480,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>104</v>
       </c>
@@ -4560,7 +4561,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="36" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>104</v>
       </c>
@@ -4641,7 +4642,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>104</v>
       </c>
@@ -4722,7 +4723,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="38" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>104</v>
       </c>
@@ -4803,7 +4804,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>104</v>
       </c>
@@ -4884,7 +4885,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>104</v>
       </c>
@@ -4965,7 +4966,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>104</v>
       </c>
@@ -5046,7 +5047,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>104</v>
       </c>
@@ -5127,7 +5128,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>104</v>
       </c>
@@ -5208,7 +5209,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="44" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>104</v>
       </c>
@@ -5289,7 +5290,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>104</v>
       </c>
@@ -5370,7 +5371,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="46" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>104</v>
       </c>
@@ -5451,7 +5452,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="47" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>104</v>
       </c>
@@ -5525,7 +5526,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="48" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>104</v>
       </c>
@@ -5606,7 +5607,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="49" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>104</v>
       </c>
@@ -5687,7 +5688,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="50" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>104</v>
       </c>
@@ -5768,7 +5769,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="51" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>104</v>
       </c>
@@ -5849,7 +5850,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="52" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>104</v>
       </c>
@@ -5930,7 +5931,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="53" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>104</v>
       </c>
@@ -6011,7 +6012,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="54" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>104</v>
       </c>
@@ -6092,7 +6093,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>104</v>
       </c>
@@ -6173,7 +6174,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="56" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>104</v>
       </c>
@@ -6254,7 +6255,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="57" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>104</v>
       </c>
@@ -6335,7 +6336,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="58" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>104</v>
       </c>
@@ -6416,7 +6417,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="59" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>104</v>
       </c>
@@ -6497,7 +6498,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="60" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>104</v>
       </c>
@@ -6578,7 +6579,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="61" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>104</v>
       </c>
@@ -6659,7 +6660,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="62" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>104</v>
       </c>
@@ -6740,7 +6741,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="63" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>104</v>
       </c>
@@ -6821,7 +6822,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="64" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>104</v>
       </c>
@@ -6902,7 +6903,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="65" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>104</v>
       </c>
@@ -6983,7 +6984,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="66" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>104</v>
       </c>
@@ -7064,7 +7065,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="67" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>104</v>
       </c>
@@ -7145,7 +7146,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="68" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>104</v>
       </c>
@@ -7226,7 +7227,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="69" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>104</v>
       </c>
@@ -7307,7 +7308,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="70" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>104</v>
       </c>
@@ -7388,7 +7389,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="71" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>104</v>
       </c>
@@ -7469,7 +7470,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="72" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>104</v>
       </c>
@@ -7550,7 +7551,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="73" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>104</v>
       </c>
@@ -7631,7 +7632,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>104</v>
       </c>
@@ -7712,7 +7713,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>104</v>
       </c>
@@ -7793,7 +7794,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>104</v>
       </c>
@@ -7874,7 +7875,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="77" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>104</v>
       </c>
@@ -7955,7 +7956,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="78" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>104</v>
       </c>
@@ -8036,7 +8037,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="79" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>104</v>
       </c>
@@ -8117,7 +8118,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="80" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>104</v>
       </c>
@@ -8198,7 +8199,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="81" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>104</v>
       </c>
@@ -8279,7 +8280,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="82" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>104</v>
       </c>
@@ -8360,7 +8361,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="83" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>104</v>
       </c>
@@ -8441,7 +8442,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="84" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>104</v>
       </c>
@@ -8522,7 +8523,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="85" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>104</v>
       </c>
@@ -8603,7 +8604,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="86" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>104</v>
       </c>
@@ -8684,7 +8685,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="87" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>104</v>
       </c>
@@ -8765,7 +8766,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="88" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>104</v>
       </c>
@@ -8846,7 +8847,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="89" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>104</v>
       </c>
@@ -8927,7 +8928,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="90" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>104</v>
       </c>
@@ -9008,7 +9009,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="91" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>104</v>
       </c>
@@ -9089,7 +9090,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="92" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>104</v>
       </c>
@@ -9170,7 +9171,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="93" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>104</v>
       </c>
@@ -9251,7 +9252,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="94" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>104</v>
       </c>
@@ -9332,7 +9333,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="95" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>104</v>
       </c>
@@ -9413,7 +9414,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="96" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>104</v>
       </c>
@@ -9494,7 +9495,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="97" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>104</v>
       </c>
@@ -9575,7 +9576,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="98" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>104</v>
       </c>
@@ -9656,7 +9657,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="99" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>104</v>
       </c>
@@ -9737,7 +9738,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="100" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>104</v>
       </c>
@@ -9818,7 +9819,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="101" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>104</v>
       </c>
@@ -9899,7 +9900,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="102" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A102" t="s">
         <v>104</v>
       </c>
@@ -9980,7 +9981,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="103" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>106</v>
       </c>
@@ -10059,7 +10060,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="104" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>106</v>
       </c>
@@ -10138,7 +10139,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="105" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>106</v>
       </c>
@@ -10217,7 +10218,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="106" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>106</v>
       </c>
@@ -10296,7 +10297,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="107" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>106</v>
       </c>
@@ -10375,7 +10376,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="108" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>106</v>
       </c>
@@ -10454,7 +10455,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="109" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>106</v>
       </c>
@@ -10533,7 +10534,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="110" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>106</v>
       </c>
@@ -10612,7 +10613,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="111" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>106</v>
       </c>
@@ -10691,7 +10692,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="112" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>106</v>
       </c>
@@ -10770,7 +10771,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="113" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
         <v>106</v>
       </c>
@@ -10849,7 +10850,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="114" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>106</v>
       </c>
@@ -10928,7 +10929,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="115" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>106</v>
       </c>
@@ -11007,7 +11008,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="116" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>106</v>
       </c>
@@ -11086,7 +11087,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="117" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>106</v>
       </c>
@@ -11165,7 +11166,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="118" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>105</v>
       </c>
@@ -11244,7 +11245,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="119" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>105</v>
       </c>
@@ -11323,7 +11324,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="120" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>105</v>
       </c>
@@ -11402,7 +11403,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="121" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
         <v>105</v>
       </c>
@@ -11481,7 +11482,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="122" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
         <v>105</v>
       </c>
@@ -11560,7 +11561,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="123" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
         <v>105</v>
       </c>
@@ -11639,7 +11640,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="124" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>105</v>
       </c>
@@ -11718,7 +11719,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="125" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
         <v>105</v>
       </c>
@@ -11797,7 +11798,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="126" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>105</v>
       </c>
@@ -11876,7 +11877,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="127" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
         <v>105</v>
       </c>
@@ -11955,7 +11956,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="128" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
         <v>105</v>
       </c>
@@ -12034,7 +12035,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="129" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
         <v>105</v>
       </c>
@@ -12113,7 +12114,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="130" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
         <v>105</v>
       </c>
@@ -12192,7 +12193,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="131" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
         <v>105</v>
       </c>
@@ -12271,7 +12272,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="132" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>105</v>
       </c>
@@ -12350,7 +12351,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="133" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
         <v>105</v>
       </c>
@@ -12429,7 +12430,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="134" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
         <v>105</v>
       </c>
@@ -12508,7 +12509,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="135" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
         <v>105</v>
       </c>
@@ -12587,7 +12588,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="136" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
         <v>105</v>
       </c>
@@ -12666,7 +12667,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="137" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
         <v>105</v>
       </c>
@@ -12745,7 +12746,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="138" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>105</v>
       </c>
@@ -12824,7 +12825,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="139" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A139" s="2"/>
       <c r="B139" s="1"/>
       <c r="C139" s="1"/>
@@ -12842,17 +12843,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DF29616-2603-4811-AA75-C70B902F2583}">
   <dimension ref="A1:H40"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="43.33203125" customWidth="1"/>
-    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.109375" customWidth="1"/>
-    <col min="4" max="4" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="43.36328125" customWidth="1"/>
+    <col min="2" max="2" width="17.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.08984375" customWidth="1"/>
+    <col min="4" max="4" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>185</v>
       </c>
@@ -12878,7 +12879,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>186</v>
       </c>
@@ -12906,7 +12907,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>103</v>
       </c>
@@ -12934,7 +12935,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>205</v>
       </c>
@@ -12962,7 +12963,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>18</v>
       </c>
@@ -12990,7 +12991,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -13018,7 +13019,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>24</v>
       </c>
@@ -13046,7 +13047,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>24</v>
       </c>
@@ -13074,7 +13075,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>187</v>
       </c>
@@ -13102,7 +13103,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -13130,7 +13131,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>34</v>
       </c>
@@ -13158,7 +13159,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>36</v>
       </c>
@@ -13186,7 +13187,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>38</v>
       </c>
@@ -13214,7 +13215,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>41</v>
       </c>
@@ -13242,7 +13243,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>44</v>
       </c>
@@ -13270,7 +13271,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>46</v>
       </c>
@@ -13298,7 +13299,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -13326,7 +13327,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>52</v>
       </c>
@@ -13354,7 +13355,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>55</v>
       </c>
@@ -13382,7 +13383,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>58</v>
       </c>
@@ -13410,7 +13411,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>60</v>
       </c>
@@ -13438,7 +13439,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>186</v>
       </c>
@@ -13466,7 +13467,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>186</v>
       </c>
@@ -13494,7 +13495,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>186</v>
       </c>
@@ -13522,7 +13523,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>186</v>
       </c>
@@ -13550,7 +13551,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>18</v>
       </c>
@@ -13578,7 +13579,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>18</v>
       </c>
@@ -13606,7 +13607,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -13634,7 +13635,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>18</v>
       </c>
@@ -13662,7 +13663,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>21</v>
       </c>
@@ -13690,7 +13691,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>21</v>
       </c>
@@ -13718,7 +13719,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>68</v>
       </c>
@@ -13746,7 +13747,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>203</v>
       </c>
@@ -13774,7 +13775,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>72</v>
       </c>
@@ -13802,7 +13803,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>74</v>
       </c>
@@ -13830,7 +13831,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>76</v>
       </c>
@@ -13858,7 +13859,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>78</v>
       </c>
@@ -13886,7 +13887,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>80</v>
       </c>
@@ -13914,7 +13915,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
         <v>82</v>
       </c>
@@ -13942,7 +13943,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
         <v>82</v>
       </c>
@@ -13978,15 +13979,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5B6FF77-C883-40C9-8616-F79923CDA0A3}">
   <dimension ref="A1:O27"/>
-  <sheetFormatPr defaultRowHeight="16.05" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.08984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>225</v>
       </c>
@@ -14033,7 +14034,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>57</v>
       </c>
@@ -14081,7 +14082,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -14120,7 +14121,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -14162,7 +14163,7 @@
         <v>-30</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>35</v>
       </c>
@@ -14210,7 +14211,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -14252,7 +14253,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>135</v>
       </c>
@@ -14282,7 +14283,7 @@
         <v>-99999</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>137</v>
       </c>
@@ -14312,7 +14313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>140</v>
       </c>
@@ -14342,7 +14343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>141</v>
       </c>
@@ -14372,7 +14373,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>142</v>
       </c>
@@ -14402,7 +14403,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>48</v>
       </c>
@@ -14441,7 +14442,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>28</v>
       </c>
@@ -14480,7 +14481,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>45</v>
       </c>
@@ -14522,7 +14523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -14555,7 +14556,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>43</v>
       </c>
@@ -14597,7 +14598,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>107</v>
       </c>
@@ -14630,7 +14631,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -14669,7 +14670,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>100</v>
       </c>
@@ -14705,7 +14706,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>31</v>
       </c>
@@ -14753,7 +14754,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -14795,7 +14796,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>17</v>
       </c>
@@ -14843,7 +14844,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>67</v>
       </c>
@@ -14882,7 +14883,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>12</v>
       </c>
@@ -14930,7 +14931,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>54</v>
       </c>
@@ -14969,7 +14970,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>51</v>
       </c>
@@ -15008,7 +15009,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
07/04/2026, CC: added tab to load csv and transform into metadata, added radio button and added shinyfiles to imports
</commit_message>
<xml_diff>
--- a/tests/testthat/data-raw/dt_meta.xlsx
+++ b/tests/testthat/data-raw/dt_meta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cehacuk-my.sharepoint.com/personal/clacap_ceh_ac_uk/Documents/metamet/tests/testthat/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{3A480153-A5CB-4962-96B3-DA1C3040D664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA9B4E97-8CB5-4EF9-BF9B-68D61D592B8D}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="13_ncr:1_{3A480153-A5CB-4962-96B3-DA1C3040D664}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E8C983C1-D57F-426A-9C3E-AF6B956C139F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
+    <workbookView xWindow="1270" yWindow="1610" windowWidth="14400" windowHeight="8170" xr2:uid="{A45171B9-DFAC-4AFC-87E9-9DEEF5646C72}"/>
   </bookViews>
   <sheets>
     <sheet name="dt_meta" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="dt_var_naming" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">dt_meta!$A$1:$X$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">dt_meta!$A$1:$X$138</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>